<commit_message>
installed python y unidades de Narea
</commit_message>
<xml_diff>
--- a/Results_isofys/Numex_preliminar_base.xlsx
+++ b/Results_isofys/Numex_preliminar_base.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BA181"/>
+  <dimension ref="A1:AZ181"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -686,11 +686,6 @@
       <c r="AZ1" s="1" t="inlineStr">
         <is>
           <t>Narea</t>
-        </is>
-      </c>
-      <c r="BA1" s="1" t="inlineStr">
-        <is>
-          <t>Carea</t>
         </is>
       </c>
     </row>
@@ -835,10 +830,7 @@
         <v>-1.069204566063425</v>
       </c>
       <c r="AZ2" t="n">
-        <v>0.1583411527786951</v>
-      </c>
-      <c r="BA2" t="n">
-        <v>6.267862957094129</v>
+        <v>1.583411527786951</v>
       </c>
     </row>
     <row r="3">
@@ -982,10 +974,7 @@
         <v>-1.162714378482783</v>
       </c>
       <c r="AZ3" t="n">
-        <v>0.1927929018543231</v>
-      </c>
-      <c r="BA3" t="n">
-        <v>4.931398966307422</v>
+        <v>1.927929018543231</v>
       </c>
     </row>
     <row r="4">
@@ -1129,10 +1118,7 @@
         <v>-1.083217188451016</v>
       </c>
       <c r="AZ4" t="n">
-        <v>0.1459443363957555</v>
-      </c>
-      <c r="BA4" t="n">
-        <v>6.201410491775166</v>
+        <v>1.459443363957554</v>
       </c>
     </row>
     <row r="5">
@@ -1276,10 +1262,7 @@
         <v>-1.173469655199274</v>
       </c>
       <c r="AZ5" t="n">
-        <v>0.2308390026071944</v>
-      </c>
-      <c r="BA5" t="n">
-        <v>6.803966990152447</v>
+        <v>2.308390026071943</v>
       </c>
     </row>
     <row r="6">
@@ -1423,10 +1406,7 @@
         <v>-1.152717050430573</v>
       </c>
       <c r="AZ6" t="n">
-        <v>0.1972952651382424</v>
-      </c>
-      <c r="BA6" t="n">
-        <v>5.814010355624786</v>
+        <v>1.972952651382424</v>
       </c>
     </row>
     <row r="7">
@@ -1570,10 +1550,7 @@
         <v>-0.9757692279498354</v>
       </c>
       <c r="AZ7" t="n">
-        <v>0.2411024955423218</v>
-      </c>
-      <c r="BA7" t="n">
-        <v>6.393667365779264</v>
+        <v>2.411024955423218</v>
       </c>
     </row>
     <row r="8">
@@ -1717,10 +1694,7 @@
         <v>-1.066817746219274</v>
       </c>
       <c r="AZ8" t="n">
-        <v>0.2212734935521185</v>
-      </c>
-      <c r="BA8" t="n">
-        <v>6.582919875238116</v>
+        <v>2.212734935521185</v>
       </c>
     </row>
     <row r="9">
@@ -1864,10 +1838,7 @@
         <v>-1.120257664680253</v>
       </c>
       <c r="AZ9" t="n">
-        <v>0.2491330280495736</v>
-      </c>
-      <c r="BA9" t="n">
-        <v>7.04653963916366</v>
+        <v>2.491330280495736</v>
       </c>
     </row>
     <row r="10">
@@ -2011,10 +1982,7 @@
         <v>-1.176763154946914</v>
       </c>
       <c r="AZ10" t="n">
-        <v>0.1922442143630735</v>
-      </c>
-      <c r="BA10" t="n">
-        <v>5.385976820401974</v>
+        <v>1.922442143630735</v>
       </c>
     </row>
     <row r="11">
@@ -2158,10 +2126,7 @@
         <v>-1.083133704760353</v>
       </c>
       <c r="AZ11" t="n">
-        <v>0.1541538771183675</v>
-      </c>
-      <c r="BA11" t="n">
-        <v>6.156964889603419</v>
+        <v>1.541538771183675</v>
       </c>
     </row>
     <row r="12">
@@ -2305,10 +2270,7 @@
         <v>-0.9693632665794485</v>
       </c>
       <c r="AZ12" t="n">
-        <v>0.1704503359635594</v>
-      </c>
-      <c r="BA12" t="n">
-        <v>7.04539122144526</v>
+        <v>1.704503359635594</v>
       </c>
     </row>
     <row r="13">
@@ -2452,10 +2414,7 @@
         <v>-1.01178671221848</v>
       </c>
       <c r="AZ13" t="n">
-        <v>0.1893086604314295</v>
-      </c>
-      <c r="BA13" t="n">
-        <v>6.298227944361334</v>
+        <v>1.893086604314296</v>
       </c>
     </row>
     <row r="14">
@@ -2599,10 +2558,7 @@
         <v>-0.9086318732906992</v>
       </c>
       <c r="AZ14" t="n">
-        <v>0.2420263723581012</v>
-      </c>
-      <c r="BA14" t="n">
-        <v>5.933547349313596</v>
+        <v>2.420263723581012</v>
       </c>
     </row>
     <row r="15">
@@ -2746,10 +2702,7 @@
         <v>-0.9710658232898745</v>
       </c>
       <c r="AZ15" t="n">
-        <v>0.2262696828216982</v>
-      </c>
-      <c r="BA15" t="n">
-        <v>6.737742901484933</v>
+        <v>2.262696828216981</v>
       </c>
     </row>
     <row r="16">
@@ -2809,7 +2762,7 @@
         <v>42.28</v>
       </c>
       <c r="P16" t="n">
-        <v>-28.2</v>
+        <v>-31.00109077040427</v>
       </c>
       <c r="Q16" t="n">
         <v>15.5</v>
@@ -2851,16 +2804,16 @@
       <c r="AJ16" t="inlineStr"/>
       <c r="AK16" t="inlineStr"/>
       <c r="AL16" t="n">
-        <v>19.32430148930667</v>
+        <v>22.27086816317477</v>
       </c>
       <c r="AM16" t="n">
-        <v>324.3159602666282</v>
+        <v>384.1537123992449</v>
       </c>
       <c r="AN16" t="n">
-        <v>0.7066443400185419</v>
+        <v>0.8370233963843873</v>
       </c>
       <c r="AO16" t="n">
-        <v>84.14763727184936</v>
+        <v>46.74904218896397</v>
       </c>
       <c r="AP16" t="n">
         <v>2000</v>
@@ -2890,13 +2843,10 @@
         <v>32.32547486872957</v>
       </c>
       <c r="AY16" t="n">
-        <v>-0.9202190103021481</v>
+        <v>-1.011623867625123</v>
       </c>
       <c r="AZ16" t="n">
-        <v>0.2346594974817987</v>
-      </c>
-      <c r="BA16" t="n">
-        <v>7.585479688556592</v>
+        <v>2.346594974817986</v>
       </c>
     </row>
     <row r="17">
@@ -3040,10 +2990,7 @@
         <v>-1.137930339273472</v>
       </c>
       <c r="AZ17" t="n">
-        <v>0.2040293659175826</v>
-      </c>
-      <c r="BA17" t="n">
-        <v>5.793309073325802</v>
+        <v>2.040293659175827</v>
       </c>
     </row>
     <row r="18">
@@ -3187,10 +3134,7 @@
         <v>-0.9983195512068304</v>
       </c>
       <c r="AZ18" t="n">
-        <v>0.2199748552043699</v>
-      </c>
-      <c r="BA18" t="n">
-        <v>6.418104834646514</v>
+        <v>2.199748552043698</v>
       </c>
     </row>
     <row r="19">
@@ -3334,10 +3278,7 @@
         <v>-1.159881181147376</v>
       </c>
       <c r="AZ19" t="n">
-        <v>0.1804095984933663</v>
-      </c>
-      <c r="BA19" t="n">
-        <v>4.811120672929789</v>
+        <v>1.804095984933663</v>
       </c>
     </row>
     <row r="20">
@@ -3397,7 +3338,7 @@
         <v>47.75</v>
       </c>
       <c r="P20" t="n">
-        <v>-26.37</v>
+        <v>-32.60541078255443</v>
       </c>
       <c r="Q20" t="n">
         <v>15.9</v>
@@ -3439,16 +3380,16 @@
       <c r="AJ20" t="inlineStr"/>
       <c r="AK20" t="inlineStr"/>
       <c r="AL20" t="n">
-        <v>17.40841612040325</v>
+        <v>23.9661945893428</v>
       </c>
       <c r="AM20" t="n">
-        <v>285.4088909524788</v>
+        <v>418.5817548299786</v>
       </c>
       <c r="AN20" t="n">
-        <v>0.6218706511290104</v>
+        <v>0.9120378400201408</v>
       </c>
       <c r="AO20" t="n">
-        <v>108.4645555931928</v>
+        <v>25.23151566975534</v>
       </c>
       <c r="AP20" t="n">
         <v>2000</v>
@@ -3478,13 +3419,10 @@
         <v>30.75436275117814</v>
       </c>
       <c r="AY20" t="n">
-        <v>-0.9251081452731393</v>
+        <v>-1.14385783446787</v>
       </c>
       <c r="AZ20" t="n">
-        <v>0.2216436966512492</v>
-      </c>
-      <c r="BA20" t="n">
-        <v>6.816510648324604</v>
+        <v>2.216436966512492</v>
       </c>
     </row>
     <row r="21">
@@ -3628,10 +3566,7 @@
         <v>-0.8250529055541557</v>
       </c>
       <c r="AZ21" t="n">
-        <v>0.2731252805030631</v>
-      </c>
-      <c r="BA21" t="n">
-        <v>6.269341168086865</v>
+        <v>2.731252805030631</v>
       </c>
     </row>
     <row r="22">
@@ -3775,10 +3710,7 @@
         <v>-0.9307778716019919</v>
       </c>
       <c r="AZ22" t="n">
-        <v>0.1359691165823957</v>
-      </c>
-      <c r="BA22" t="n">
-        <v>7.209869586996444</v>
+        <v>1.359691165823957</v>
       </c>
     </row>
     <row r="23">
@@ -3922,10 +3854,7 @@
         <v>-1.076624094600751</v>
       </c>
       <c r="AZ23" t="n">
-        <v>0.1532285064088778</v>
-      </c>
-      <c r="BA23" t="n">
-        <v>5.8814772925756</v>
+        <v>1.532285064088778</v>
       </c>
     </row>
     <row r="24">
@@ -4069,10 +3998,7 @@
         <v>-0.9531215121310557</v>
       </c>
       <c r="AZ24" t="n">
-        <v>0.2083919474390169</v>
-      </c>
-      <c r="BA24" t="n">
-        <v>6.450269324889292</v>
+        <v>2.083919474390169</v>
       </c>
     </row>
     <row r="25">
@@ -4216,10 +4142,7 @@
         <v>-1.127672428671739</v>
       </c>
       <c r="AZ25" t="n">
-        <v>0.1924962019984864</v>
-      </c>
-      <c r="BA25" t="n">
-        <v>5.922628309595306</v>
+        <v>1.924962019984864</v>
       </c>
     </row>
     <row r="26">
@@ -4363,10 +4286,7 @@
         <v>-1.093730835683608</v>
       </c>
       <c r="AZ26" t="n">
-        <v>0.1993680458705612</v>
-      </c>
-      <c r="BA26" t="n">
-        <v>5.819873982352418</v>
+        <v>1.993680458705612</v>
       </c>
     </row>
     <row r="27">
@@ -4510,10 +4430,7 @@
         <v>-0.9251981278059437</v>
       </c>
       <c r="AZ27" t="n">
-        <v>0.2247906864753312</v>
-      </c>
-      <c r="BA27" t="n">
-        <v>4.353630630525455</v>
+        <v>2.247906864753312</v>
       </c>
     </row>
     <row r="28">
@@ -4657,10 +4574,7 @@
         <v>-1.110646754176239</v>
       </c>
       <c r="AZ28" t="n">
-        <v>0.1941969337398241</v>
-      </c>
-      <c r="BA28" t="n">
-        <v>6.180318961158282</v>
+        <v>1.941969337398241</v>
       </c>
     </row>
     <row r="29">
@@ -4804,10 +4718,7 @@
         <v>-0.8721981465115956</v>
       </c>
       <c r="AZ29" t="n">
-        <v>0.2299853817964811</v>
-      </c>
-      <c r="BA29" t="n">
-        <v>4.77039521233669</v>
+        <v>2.299853817964811</v>
       </c>
     </row>
     <row r="30">
@@ -4951,10 +4862,7 @@
         <v>-1.026018023099852</v>
       </c>
       <c r="AZ30" t="n">
-        <v>0.2056480718564838</v>
-      </c>
-      <c r="BA30" t="n">
-        <v>6.003256549989229</v>
+        <v>2.056480718564837</v>
       </c>
     </row>
     <row r="31">
@@ -5098,10 +5006,7 @@
         <v>-1.081725628636109</v>
       </c>
       <c r="AZ31" t="n">
-        <v>0.136631885562437</v>
-      </c>
-      <c r="BA31" t="n">
-        <v>5.871422404388254</v>
+        <v>1.36631885562437</v>
       </c>
     </row>
     <row r="32">
@@ -5245,10 +5150,7 @@
         <v>-0.9757257325131097</v>
       </c>
       <c r="AZ32" t="n">
-        <v>0.2060536274187499</v>
-      </c>
-      <c r="BA32" t="n">
-        <v>4.248872527334292</v>
+        <v>2.060536274187499</v>
       </c>
     </row>
     <row r="33">
@@ -5392,10 +5294,7 @@
         <v>-1.108000186694067</v>
       </c>
       <c r="AZ33" t="n">
-        <v>0.2140487849336566</v>
-      </c>
-      <c r="BA33" t="n">
-        <v>4.707179999838402</v>
+        <v>2.140487849336566</v>
       </c>
     </row>
     <row r="34">
@@ -5539,10 +5438,7 @@
         <v>-1.1317622997201</v>
       </c>
       <c r="AZ34" t="n">
-        <v>0.1262484116656832</v>
-      </c>
-      <c r="BA34" t="n">
-        <v>5.538752547725021</v>
+        <v>1.262484116656831</v>
       </c>
     </row>
     <row r="35">
@@ -5686,10 +5582,7 @@
         <v>-1.097985206987246</v>
       </c>
       <c r="AZ35" t="n">
-        <v>0.236853606683806</v>
-      </c>
-      <c r="BA35" t="n">
-        <v>5.72708070874746</v>
+        <v>2.36853606683806</v>
       </c>
     </row>
     <row r="36">
@@ -5833,10 +5726,7 @@
         <v>-1.041003254864917</v>
       </c>
       <c r="AZ36" t="n">
-        <v>0.1404492354378129</v>
-      </c>
-      <c r="BA36" t="n">
-        <v>6.421580057406096</v>
+        <v>1.404492354378129</v>
       </c>
     </row>
     <row r="37">
@@ -5980,10 +5870,7 @@
         <v>-1.128326182974303</v>
       </c>
       <c r="AZ37" t="n">
-        <v>0.165736668134432</v>
-      </c>
-      <c r="BA37" t="n">
-        <v>5.382476778431748</v>
+        <v>1.65736668134432</v>
       </c>
     </row>
     <row r="38">
@@ -6127,10 +6014,7 @@
         <v>-1.052221717593601</v>
       </c>
       <c r="AZ38" t="n">
-        <v>0.25370946862891</v>
-      </c>
-      <c r="BA38" t="n">
-        <v>7.926449640071605</v>
+        <v>2.5370946862891</v>
       </c>
     </row>
     <row r="39">
@@ -6274,10 +6158,7 @@
         <v>-1.018263130425242</v>
       </c>
       <c r="AZ39" t="n">
-        <v>0.1790085898974969</v>
-      </c>
-      <c r="BA39" t="n">
-        <v>3.990234824028318</v>
+        <v>1.790085898974969</v>
       </c>
     </row>
     <row r="40">
@@ -6421,10 +6302,7 @@
         <v>-1.134852638614013</v>
       </c>
       <c r="AZ40" t="n">
-        <v>0.1636334848571583</v>
-      </c>
-      <c r="BA40" t="n">
-        <v>6.701960533465813</v>
+        <v>1.636334848571583</v>
       </c>
     </row>
     <row r="41">
@@ -6568,10 +6446,7 @@
         <v>-1.046794083447492</v>
       </c>
       <c r="AZ41" t="n">
-        <v>0.1962293560349081</v>
-      </c>
-      <c r="BA41" t="n">
-        <v>6.406993482654983</v>
+        <v>1.962293560349081</v>
       </c>
     </row>
     <row r="42">
@@ -6715,10 +6590,7 @@
         <v>-1.055363556422817</v>
       </c>
       <c r="AZ42" t="n">
-        <v>0.1962293560349081</v>
-      </c>
-      <c r="BA42" t="n">
-        <v>6.406993482654983</v>
+        <v>1.962293560349081</v>
       </c>
     </row>
     <row r="43">
@@ -6862,10 +6734,7 @@
         <v>-1.027478472194354</v>
       </c>
       <c r="AZ43" t="n">
-        <v>0.1962293560349081</v>
-      </c>
-      <c r="BA43" t="n">
-        <v>6.406993482654983</v>
+        <v>1.962293560349081</v>
       </c>
     </row>
     <row r="44">
@@ -7009,10 +6878,7 @@
         <v>-1.035889819888641</v>
       </c>
       <c r="AZ44" t="n">
-        <v>0.1962293560349081</v>
-      </c>
-      <c r="BA44" t="n">
-        <v>6.406993482654983</v>
+        <v>1.962293560349081</v>
       </c>
     </row>
     <row r="45">
@@ -7156,10 +7022,7 @@
         <v>-1.016944806660762</v>
       </c>
       <c r="AZ45" t="n">
-        <v>0.2080347916779913</v>
-      </c>
-      <c r="BA45" t="n">
-        <v>7.270477607848516</v>
+        <v>2.080347916779913</v>
       </c>
     </row>
     <row r="46">
@@ -7303,10 +7166,7 @@
         <v>-1.168428613749502</v>
       </c>
       <c r="AZ46" t="n">
-        <v>0.1803572361821152</v>
-      </c>
-      <c r="BA46" t="n">
-        <v>4.981358951370535</v>
+        <v>1.803572361821152</v>
       </c>
     </row>
     <row r="47">
@@ -7450,10 +7310,7 @@
         <v>-1.006406074511895</v>
       </c>
       <c r="AZ47" t="n">
-        <v>0.1563233988308393</v>
-      </c>
-      <c r="BA47" t="n">
-        <v>4.941560931653564</v>
+        <v>1.563233988308393</v>
       </c>
     </row>
     <row r="48">
@@ -7597,10 +7454,7 @@
         <v>-1.002974473340656</v>
       </c>
       <c r="AZ48" t="n">
-        <v>0.1727182447385554</v>
-      </c>
-      <c r="BA48" t="n">
-        <v>5.627608137299266</v>
+        <v>1.727182447385554</v>
       </c>
     </row>
     <row r="49">
@@ -7744,10 +7598,7 @@
         <v>-1.033343565098957</v>
       </c>
       <c r="AZ49" t="n">
-        <v>0.2118768969038876</v>
-      </c>
-      <c r="BA49" t="n">
-        <v>7.860992204916545</v>
+        <v>2.118768969038876</v>
       </c>
     </row>
     <row r="50">
@@ -7891,10 +7742,7 @@
         <v>-1.094831536193773</v>
       </c>
       <c r="AZ50" t="n">
-        <v>0.1305405133948935</v>
-      </c>
-      <c r="BA50" t="n">
-        <v>6.085878779925097</v>
+        <v>1.305405133948935</v>
       </c>
     </row>
     <row r="51">
@@ -8038,10 +7886,7 @@
         <v>-1.034130614924995</v>
       </c>
       <c r="AZ51" t="n">
-        <v>0.2749705279828398</v>
-      </c>
-      <c r="BA51" t="n">
-        <v>7.600880368696366</v>
+        <v>2.749705279828397</v>
       </c>
     </row>
     <row r="52">
@@ -8185,10 +8030,7 @@
         <v>-0.9330413776996519</v>
       </c>
       <c r="AZ52" t="n">
-        <v>0.2554237568151246</v>
-      </c>
-      <c r="BA52" t="n">
-        <v>8.029662939995131</v>
+        <v>2.554237568151246</v>
       </c>
     </row>
     <row r="53">
@@ -8232,9 +8074,7 @@
       <c r="J53" t="n">
         <v>-32.30627681984863</v>
       </c>
-      <c r="K53" t="n">
-        <v>0.0253654953216571</v>
-      </c>
+      <c r="K53" t="inlineStr"/>
       <c r="L53" t="n">
         <v>2.212395175186674</v>
       </c>
@@ -8325,18 +8165,11 @@
       <c r="AW53" t="n">
         <v>0.5561426684280054</v>
       </c>
-      <c r="AX53" t="n">
-        <v>16.47515809594595</v>
-      </c>
+      <c r="AX53" t="inlineStr"/>
       <c r="AY53" t="n">
         <v>-1.059704205037399</v>
       </c>
-      <c r="AZ53" t="n">
-        <v>0.2105696461538427</v>
-      </c>
-      <c r="BA53" t="n">
-        <v>3.469168210591955</v>
-      </c>
+      <c r="AZ53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="1" t="n">
@@ -8479,10 +8312,7 @@
         <v>-1.09799079624996</v>
       </c>
       <c r="AZ54" t="n">
-        <v>0.2230482700063978</v>
-      </c>
-      <c r="BA54" t="n">
-        <v>3.834114387266885</v>
+        <v>2.230482700063977</v>
       </c>
     </row>
     <row r="55">
@@ -8626,10 +8456,7 @@
         <v>-1.013558134662488</v>
       </c>
       <c r="AZ55" t="n">
-        <v>0.2700331914670088</v>
-      </c>
-      <c r="BA55" t="n">
-        <v>9.226808188432537</v>
+        <v>2.700331914670088</v>
       </c>
     </row>
     <row r="56">
@@ -8773,10 +8600,7 @@
         <v>-1.029758709416929</v>
       </c>
       <c r="AZ56" t="n">
-        <v>0.1811914954031918</v>
-      </c>
-      <c r="BA56" t="n">
-        <v>5.640759522824799</v>
+        <v>1.811914954031917</v>
       </c>
     </row>
     <row r="57">
@@ -8920,10 +8744,7 @@
         <v>-1.071407723597514</v>
       </c>
       <c r="AZ57" t="n">
-        <v>0.1485071659290358</v>
-      </c>
-      <c r="BA57" t="n">
-        <v>6.279270830799232</v>
+        <v>1.485071659290358</v>
       </c>
     </row>
     <row r="58">
@@ -9067,10 +8888,7 @@
         <v>-1.076020463092165</v>
       </c>
       <c r="AZ58" t="n">
-        <v>0.181805467668072</v>
-      </c>
-      <c r="BA58" t="n">
-        <v>5.528408572483942</v>
+        <v>1.818054676680719</v>
       </c>
     </row>
     <row r="59">
@@ -9214,10 +9032,7 @@
         <v>-1.131721301339614</v>
       </c>
       <c r="AZ59" t="n">
-        <v>0.1468960643433882</v>
-      </c>
-      <c r="BA59" t="n">
-        <v>6.080598725084783</v>
+        <v>1.468960643433882</v>
       </c>
     </row>
     <row r="60">
@@ -9361,10 +9176,7 @@
         <v>-1.148906986345209</v>
       </c>
       <c r="AZ60" t="n">
-        <v>0.1640718941643498</v>
-      </c>
-      <c r="BA60" t="n">
-        <v>4.620440023861259</v>
+        <v>1.640718941643499</v>
       </c>
     </row>
     <row r="61">
@@ -9508,10 +9320,7 @@
         <v>-0.9802187884414533</v>
       </c>
       <c r="AZ61" t="n">
-        <v>0.2324436326842925</v>
-      </c>
-      <c r="BA61" t="n">
-        <v>6.589693642640406</v>
+        <v>2.324436326842925</v>
       </c>
     </row>
     <row r="62">
@@ -9655,10 +9464,7 @@
         <v>-1.059967417806882</v>
       </c>
       <c r="AZ62" t="n">
-        <v>0.2271852849396293</v>
-      </c>
-      <c r="BA62" t="n">
-        <v>8.1219991100984</v>
+        <v>2.271852849396293</v>
       </c>
     </row>
     <row r="63">
@@ -9802,10 +9608,7 @@
         <v>-1.07072599241777</v>
       </c>
       <c r="AZ63" t="n">
-        <v>0.2097736888129386</v>
-      </c>
-      <c r="BA63" t="n">
-        <v>6.659317142649229</v>
+        <v>2.097736888129386</v>
       </c>
     </row>
     <row r="64">
@@ -9949,10 +9752,7 @@
         <v>-1.07072599241777</v>
       </c>
       <c r="AZ64" t="n">
-        <v>0.2051731480905204</v>
-      </c>
-      <c r="BA64" t="n">
-        <v>6.720409857723063</v>
+        <v>2.051731480905203</v>
       </c>
     </row>
     <row r="65">
@@ -10096,10 +9896,7 @@
         <v>-1.072717162486702</v>
       </c>
       <c r="AZ65" t="n">
-        <v>0.1711270057226029</v>
-      </c>
-      <c r="BA65" t="n">
-        <v>6.465141386759904</v>
+        <v>1.71127005722603</v>
       </c>
     </row>
     <row r="66">
@@ -10243,10 +10040,7 @@
         <v>-1.186907968195777</v>
       </c>
       <c r="AZ66" t="n">
-        <v>0.1264668813853405</v>
-      </c>
-      <c r="BA66" t="n">
-        <v>5.917373389442116</v>
+        <v>1.264668813853404</v>
       </c>
     </row>
     <row r="67">
@@ -10390,10 +10184,7 @@
         <v>-1.05716724908219</v>
       </c>
       <c r="AZ67" t="n">
-        <v>0.1735620252135451</v>
-      </c>
-      <c r="BA67" t="n">
-        <v>5.130229695978934</v>
+        <v>1.735620252135451</v>
       </c>
     </row>
     <row r="68">
@@ -10537,10 +10328,7 @@
         <v>-1.062612342442872</v>
       </c>
       <c r="AZ68" t="n">
-        <v>0.1651892043876882</v>
-      </c>
-      <c r="BA68" t="n">
-        <v>4.61721716535054</v>
+        <v>1.651892043876882</v>
       </c>
     </row>
     <row r="69">
@@ -10684,10 +10472,7 @@
         <v>-1.162202419950019</v>
       </c>
       <c r="AZ69" t="n">
-        <v>0.1729739026459769</v>
-      </c>
-      <c r="BA69" t="n">
-        <v>4.169261023831525</v>
+        <v>1.72973902645977</v>
       </c>
     </row>
     <row r="70">
@@ -10831,10 +10616,7 @@
         <v>-0.9735100220183867</v>
       </c>
       <c r="AZ70" t="n">
-        <v>0.1653302877966243</v>
-      </c>
-      <c r="BA70" t="n">
-        <v>5.468910140257988</v>
+        <v>1.653302877966243</v>
       </c>
     </row>
     <row r="71">
@@ -10978,10 +10760,7 @@
         <v>-1.151540486656524</v>
       </c>
       <c r="AZ71" t="n">
-        <v>0.224534879706159</v>
-      </c>
-      <c r="BA71" t="n">
-        <v>6.385261085941602</v>
+        <v>2.24534879706159</v>
       </c>
     </row>
     <row r="72">
@@ -11125,10 +10904,7 @@
         <v>-1.081507885923864</v>
       </c>
       <c r="AZ72" t="n">
-        <v>0.1704181532420173</v>
-      </c>
-      <c r="BA72" t="n">
-        <v>4.64552151410903</v>
+        <v>1.704181532420173</v>
       </c>
     </row>
     <row r="73">
@@ -11272,10 +11048,7 @@
         <v>-1.008164398010397</v>
       </c>
       <c r="AZ73" t="n">
-        <v>0.1771344004138958</v>
-      </c>
-      <c r="BA73" t="n">
-        <v>5.317720031155273</v>
+        <v>1.771344004138958</v>
       </c>
     </row>
     <row r="74">
@@ -11419,10 +11192,7 @@
         <v>-0.9019527661726316</v>
       </c>
       <c r="AZ74" t="n">
-        <v>0.2890653446677475</v>
-      </c>
-      <c r="BA74" t="n">
-        <v>7.650714677495467</v>
+        <v>2.890653446677475</v>
       </c>
     </row>
     <row r="75">
@@ -11566,10 +11336,7 @@
         <v>-1.064321440481539</v>
       </c>
       <c r="AZ75" t="n">
-        <v>0.2678379030470969</v>
-      </c>
-      <c r="BA75" t="n">
-        <v>8.094394089102797</v>
+        <v>2.678379030470969</v>
       </c>
     </row>
     <row r="76">
@@ -11713,10 +11480,7 @@
         <v>-1.036430349351861</v>
       </c>
       <c r="AZ76" t="n">
-        <v>0.2020516390549202</v>
-      </c>
-      <c r="BA76" t="n">
-        <v>6.613829372688381</v>
+        <v>2.020516390549202</v>
       </c>
     </row>
     <row r="77">
@@ -11860,10 +11624,7 @@
         <v>-0.9447135609596995</v>
       </c>
       <c r="AZ77" t="n">
-        <v>0.2290004233178914</v>
-      </c>
-      <c r="BA77" t="n">
-        <v>6.379856596163442</v>
+        <v>2.290004233178915</v>
       </c>
     </row>
     <row r="78">
@@ -12007,10 +11768,7 @@
         <v>-1.136069687512091</v>
       </c>
       <c r="AZ78" t="n">
-        <v>0.2143935207599353</v>
-      </c>
-      <c r="BA78" t="n">
-        <v>4.677253989798563</v>
+        <v>2.143935207599353</v>
       </c>
     </row>
     <row r="79">
@@ -12154,10 +11912,7 @@
         <v>-0.7957323640055816</v>
       </c>
       <c r="AZ79" t="n">
-        <v>0.3250436485054538</v>
-      </c>
-      <c r="BA79" t="n">
-        <v>5.943353709831833</v>
+        <v>3.250436485054538</v>
       </c>
     </row>
     <row r="80">
@@ -12301,10 +12056,7 @@
         <v>-1.083830924468203</v>
       </c>
       <c r="AZ80" t="n">
-        <v>0.2998648154876037</v>
-      </c>
-      <c r="BA80" t="n">
-        <v>6.635735356277657</v>
+        <v>2.998648154876038</v>
       </c>
     </row>
     <row r="81">
@@ -12448,10 +12200,7 @@
         <v>-0.852490835998494</v>
       </c>
       <c r="AZ81" t="n">
-        <v>0.2994186256562353</v>
-      </c>
-      <c r="BA81" t="n">
-        <v>7.152431113667959</v>
+        <v>2.994186256562354</v>
       </c>
     </row>
     <row r="82">
@@ -12595,10 +12344,7 @@
         <v>-1.073512489772441</v>
       </c>
       <c r="AZ82" t="n">
-        <v>0.1986099449474032</v>
-      </c>
-      <c r="BA82" t="n">
-        <v>5.80366638296212</v>
+        <v>1.986099449474032</v>
       </c>
     </row>
     <row r="83">
@@ -12742,10 +12488,7 @@
         <v>-1.045162407612312</v>
       </c>
       <c r="AZ83" t="n">
-        <v>0.1574768288150041</v>
-      </c>
-      <c r="BA83" t="n">
-        <v>4.144199615258708</v>
+        <v>1.574768288150041</v>
       </c>
     </row>
     <row r="84">
@@ -12889,10 +12632,7 @@
         <v>-1.011763599487811</v>
       </c>
       <c r="AZ84" t="n">
-        <v>0.1625698637855855</v>
-      </c>
-      <c r="BA84" t="n">
-        <v>4.910286937521602</v>
+        <v>1.625698637855855</v>
       </c>
     </row>
     <row r="85">
@@ -13036,10 +12776,7 @@
         <v>-1.056436243301099</v>
       </c>
       <c r="AZ85" t="n">
-        <v>0.2261410104794487</v>
-      </c>
-      <c r="BA85" t="n">
-        <v>6.328175428570905</v>
+        <v>2.261410104794487</v>
       </c>
     </row>
     <row r="86">
@@ -13183,10 +12920,7 @@
         <v>-1.139184969499528</v>
       </c>
       <c r="AZ86" t="n">
-        <v>0.2131678007547578</v>
-      </c>
-      <c r="BA86" t="n">
-        <v>6.522638295327906</v>
+        <v>2.131678007547578</v>
       </c>
     </row>
     <row r="87">
@@ -13330,10 +13064,7 @@
         <v>-0.9994064701242487</v>
       </c>
       <c r="AZ87" t="n">
-        <v>0.2723142473493239</v>
-      </c>
-      <c r="BA87" t="n">
-        <v>7.354363492686352</v>
+        <v>2.723142473493239</v>
       </c>
     </row>
     <row r="88">
@@ -13477,10 +13208,7 @@
         <v>-0.9530514877786842</v>
       </c>
       <c r="AZ88" t="n">
-        <v>0.2165437559626953</v>
-      </c>
-      <c r="BA88" t="n">
-        <v>4.352489670002637</v>
+        <v>2.165437559626953</v>
       </c>
     </row>
     <row r="89">
@@ -13646,10 +13374,7 @@
         <v>-0.921325744894543</v>
       </c>
       <c r="AZ89" t="n">
-        <v>0.2273110803333757</v>
-      </c>
-      <c r="BA89" t="n">
-        <v>13.49936057389324</v>
+        <v>2.273110803333757</v>
       </c>
     </row>
     <row r="90">
@@ -13815,10 +13540,7 @@
         <v>-0.9396264176117411</v>
       </c>
       <c r="AZ90" t="n">
-        <v>0.2562349769016561</v>
-      </c>
-      <c r="BA90" t="n">
-        <v>14.11226797838226</v>
+        <v>2.562349769016562</v>
       </c>
     </row>
     <row r="91">
@@ -13984,10 +13706,7 @@
         <v>-0.9000000000000001</v>
       </c>
       <c r="AZ91" t="n">
-        <v>0.2747689268163115</v>
-      </c>
-      <c r="BA91" t="n">
-        <v>12.41339472150039</v>
+        <v>2.747689268163116</v>
       </c>
     </row>
     <row r="92">
@@ -14153,10 +13872,7 @@
         <v>-0.9772876892692561</v>
       </c>
       <c r="AZ92" t="n">
-        <v>0.2638257036105743</v>
-      </c>
-      <c r="BA92" t="n">
-        <v>11.44644073918296</v>
+        <v>2.638257036105744</v>
       </c>
     </row>
     <row r="93">
@@ -14322,10 +14038,7 @@
         <v>-0.8726919339164237</v>
       </c>
       <c r="AZ93" t="n">
-        <v>0.2205905999210828</v>
-      </c>
-      <c r="BA93" t="n">
-        <v>13.46108772447198</v>
+        <v>2.205905999210828</v>
       </c>
     </row>
     <row r="94">
@@ -14491,10 +14204,7 @@
         <v>-0.8030209617755858</v>
       </c>
       <c r="AZ94" t="n">
-        <v>0.2899244513121407</v>
-      </c>
-      <c r="BA94" t="n">
-        <v>14.55098595795598</v>
+        <v>2.899244513121407</v>
       </c>
     </row>
     <row r="95">
@@ -14660,10 +14370,7 @@
         <v>-0.9410150891632374</v>
       </c>
       <c r="AZ95" t="n">
-        <v>0.3639814907180162</v>
-      </c>
-      <c r="BA95" t="n">
-        <v>16.21005166131244</v>
+        <v>3.639814907180162</v>
       </c>
     </row>
     <row r="96">
@@ -14829,10 +14536,7 @@
         <v>-0.8697027197975964</v>
       </c>
       <c r="AZ96" t="n">
-        <v>0.2754165199655664</v>
-      </c>
-      <c r="BA96" t="n">
-        <v>11.5432612977339</v>
+        <v>2.754165199655663</v>
       </c>
     </row>
     <row r="97">
@@ -14998,10 +14702,7 @@
         <v>-0.8926196808510639</v>
       </c>
       <c r="AZ97" t="n">
-        <v>0.2635851161810385</v>
-      </c>
-      <c r="BA97" t="n">
-        <v>18.63708247181081</v>
+        <v>2.635851161810386</v>
       </c>
     </row>
     <row r="98">
@@ -15167,10 +14868,7 @@
         <v>-0.9120214909335124</v>
       </c>
       <c r="AZ98" t="n">
-        <v>0.2379812101557392</v>
-      </c>
-      <c r="BA98" t="n">
-        <v>13.36431271950471</v>
+        <v>2.379812101557392</v>
       </c>
     </row>
     <row r="99">
@@ -15336,10 +15034,7 @@
         <v>-0.9579330904272938</v>
       </c>
       <c r="AZ99" t="n">
-        <v>0.1937192235493845</v>
-      </c>
-      <c r="BA99" t="n">
-        <v>10.8080729022015</v>
+        <v>1.937192235493844</v>
       </c>
     </row>
     <row r="100">
@@ -15505,10 +15200,7 @@
         <v>-0.8845169545745361</v>
       </c>
       <c r="AZ100" t="n">
-        <v>0.1937567807703534</v>
-      </c>
-      <c r="BA100" t="n">
-        <v>12.77530493515518</v>
+        <v>1.937567807703533</v>
       </c>
     </row>
     <row r="101">
@@ -15674,10 +15366,7 @@
         <v>-0.8345370978332239</v>
       </c>
       <c r="AZ101" t="n">
-        <v>0.2390186769233919</v>
-      </c>
-      <c r="BA101" t="n">
-        <v>14.95225993840202</v>
+        <v>2.390186769233919</v>
       </c>
     </row>
     <row r="102">
@@ -15843,10 +15532,7 @@
         <v>-0.8655913978494624</v>
       </c>
       <c r="AZ102" t="n">
-        <v>0.3022826134073608</v>
-      </c>
-      <c r="BA102" t="n">
-        <v>14.56543934132861</v>
+        <v>3.022826134073608</v>
       </c>
     </row>
     <row r="103">
@@ -16012,10 +15698,7 @@
         <v>-0.8713188220230473</v>
       </c>
       <c r="AZ103" t="n">
-        <v>0.2697981424651091</v>
-      </c>
-      <c r="BA103" t="n">
-        <v>13.085308400592</v>
+        <v>2.697981424651091</v>
       </c>
     </row>
     <row r="104">
@@ -16181,10 +15864,7 @@
         <v>-0.873405299313052</v>
       </c>
       <c r="AZ104" t="n">
-        <v>0.3273385634947573</v>
-      </c>
-      <c r="BA104" t="n">
-        <v>13.77626263997392</v>
+        <v>3.273385634947574</v>
       </c>
     </row>
     <row r="105">
@@ -16350,10 +16030,7 @@
         <v>-0.7809629835791817</v>
       </c>
       <c r="AZ105" t="n">
-        <v>0.2627407067212578</v>
-      </c>
-      <c r="BA105" t="n">
-        <v>13.64813509985642</v>
+        <v>2.627407067212578</v>
       </c>
     </row>
     <row r="106">
@@ -16519,10 +16196,7 @@
         <v>-0.9106683804627249</v>
       </c>
       <c r="AZ106" t="n">
-        <v>0.2253565398386968</v>
-      </c>
-      <c r="BA106" t="n">
-        <v>12.53521760130511</v>
+        <v>2.253565398386967</v>
       </c>
     </row>
     <row r="107">
@@ -16688,10 +16362,7 @@
         <v>-0.840602950609365</v>
       </c>
       <c r="AZ107" t="n">
-        <v>0.2310070069738794</v>
-      </c>
-      <c r="BA107" t="n">
-        <v>13.61822728292262</v>
+        <v>2.310070069738794</v>
       </c>
     </row>
     <row r="108">
@@ -16857,10 +16528,7 @@
         <v>-0.9048231511254019</v>
       </c>
       <c r="AZ108" t="n">
-        <v>0.2004180823301927</v>
-      </c>
-      <c r="BA108" t="n">
-        <v>12.36377526016233</v>
+        <v>2.004180823301927</v>
       </c>
     </row>
     <row r="109">
@@ -17026,10 +16694,7 @@
         <v>-0.8401015228426396</v>
       </c>
       <c r="AZ109" t="n">
-        <v>0.3164054433208752</v>
-      </c>
-      <c r="BA109" t="n">
-        <v>13.4521818706214</v>
+        <v>3.164054433208753</v>
       </c>
     </row>
     <row r="110">
@@ -17195,10 +16860,7 @@
         <v>-0.9122807017543859</v>
       </c>
       <c r="AZ110" t="n">
-        <v>0.3143298872640892</v>
-      </c>
-      <c r="BA110" t="n">
-        <v>13.71728615868613</v>
+        <v>3.143298872640891</v>
       </c>
     </row>
     <row r="111">
@@ -17364,10 +17026,7 @@
         <v>-0.9649181423321083</v>
       </c>
       <c r="AZ111" t="n">
-        <v>0.2727743536270423</v>
-      </c>
-      <c r="BA111" t="n">
-        <v>13.16711084989783</v>
+        <v>2.727743536270423</v>
       </c>
     </row>
     <row r="112">
@@ -17533,10 +17192,7 @@
         <v>-0.9372869802317655</v>
       </c>
       <c r="AZ112" t="n">
-        <v>0.2677287744794695</v>
-      </c>
-      <c r="BA112" t="n">
-        <v>14.90856583514423</v>
+        <v>2.677287744794695</v>
       </c>
     </row>
     <row r="113">
@@ -17702,10 +17358,7 @@
         <v>-0.8688741721854304</v>
       </c>
       <c r="AZ113" t="n">
-        <v>0.2699350840327465</v>
-      </c>
-      <c r="BA113" t="n">
-        <v>12.56625000971446</v>
+        <v>2.699350840327465</v>
       </c>
     </row>
     <row r="114">
@@ -17871,10 +17524,7 @@
         <v>-0.821639344262295</v>
       </c>
       <c r="AZ114" t="n">
-        <v>0.4709552277566549</v>
-      </c>
-      <c r="BA114" t="n">
-        <v>13.55543529737596</v>
+        <v>4.70955227756655</v>
       </c>
     </row>
     <row r="115">
@@ -18040,10 +17690,7 @@
         <v>-1.043353636689359</v>
       </c>
       <c r="AZ115" t="n">
-        <v>0.3439129986152255</v>
-      </c>
-      <c r="BA115" t="n">
-        <v>13.8462674929608</v>
+        <v>3.439129986152254</v>
       </c>
     </row>
     <row r="116">
@@ -18209,10 +17856,7 @@
         <v>-1.023550087873462</v>
       </c>
       <c r="AZ116" t="n">
-        <v>0.3494573532195661</v>
-      </c>
-      <c r="BA116" t="n">
-        <v>14.06948853210919</v>
+        <v>3.494573532195661</v>
       </c>
     </row>
     <row r="117">
@@ -18378,10 +18022,7 @@
         <v>-0.9992862241256246</v>
       </c>
       <c r="AZ117" t="n">
-        <v>0.2941786834792475</v>
-      </c>
-      <c r="BA117" t="n">
-        <v>11.36362404621276</v>
+        <v>2.941786834792475</v>
       </c>
     </row>
     <row r="118">
@@ -18547,10 +18188,7 @@
         <v>-0.9220733427362482</v>
       </c>
       <c r="AZ118" t="n">
-        <v>0.2356234081045346</v>
-      </c>
-      <c r="BA118" t="n">
-        <v>11.21671934408004</v>
+        <v>2.356234081045346</v>
       </c>
     </row>
     <row r="119">
@@ -18716,10 +18354,7 @@
         <v>-0.9540313754104341</v>
       </c>
       <c r="AZ119" t="n">
-        <v>0.2664652002443708</v>
-      </c>
-      <c r="BA119" t="n">
-        <v>12.68492545010291</v>
+        <v>2.664652002443708</v>
       </c>
     </row>
     <row r="120">
@@ -18885,10 +18520,7 @@
         <v>-0.8568159529257928</v>
       </c>
       <c r="AZ120" t="n">
-        <v>0.4458705469717965</v>
-      </c>
-      <c r="BA120" t="n">
-        <v>16.98593273105596</v>
+        <v>4.458705469717965</v>
       </c>
     </row>
     <row r="121">
@@ -19054,10 +18686,7 @@
         <v>-0.8646491519787163</v>
       </c>
       <c r="AZ121" t="n">
-        <v>0.4809162989997219</v>
-      </c>
-      <c r="BA121" t="n">
-        <v>17.24069091284437</v>
+        <v>4.809162989997219</v>
       </c>
     </row>
     <row r="122">
@@ -19223,10 +18852,7 @@
         <v>-0.8040981061782054</v>
       </c>
       <c r="AZ122" t="n">
-        <v>0.2754411937467637</v>
-      </c>
-      <c r="BA122" t="n">
-        <v>12.9142850910087</v>
+        <v>2.754411937467637</v>
       </c>
     </row>
     <row r="123">
@@ -19392,10 +19018,7 @@
         <v>-0.9652323580034423</v>
       </c>
       <c r="AZ123" t="n">
-        <v>0.2712645733328085</v>
-      </c>
-      <c r="BA123" t="n">
-        <v>13.89093963768983</v>
+        <v>2.712645733328085</v>
       </c>
     </row>
     <row r="124">
@@ -19561,10 +19184,7 @@
         <v>-0.9461077844311376</v>
       </c>
       <c r="AZ124" t="n">
-        <v>0.3551411071187895</v>
-      </c>
-      <c r="BA124" t="n">
-        <v>15.89478030353562</v>
+        <v>3.551411071187895</v>
       </c>
     </row>
     <row r="125">
@@ -19730,10 +19350,7 @@
         <v>-0.9985683607730851</v>
       </c>
       <c r="AZ125" t="n">
-        <v>0.307205325190028</v>
-      </c>
-      <c r="BA125" t="n">
-        <v>11.82301848502743</v>
+        <v>3.07205325190028</v>
       </c>
     </row>
     <row r="126">
@@ -19899,10 +19516,7 @@
         <v>-0.8554932365555923</v>
       </c>
       <c r="AZ126" t="n">
-        <v>0.3403595277379776</v>
-      </c>
-      <c r="BA126" t="n">
-        <v>12.94346879140066</v>
+        <v>3.403595277379776</v>
       </c>
     </row>
     <row r="127">
@@ -20068,10 +19682,7 @@
         <v>-0.8341742347796839</v>
       </c>
       <c r="AZ127" t="n">
-        <v>0.3160063990834164</v>
-      </c>
-      <c r="BA127" t="n">
-        <v>13.49082394850428</v>
+        <v>3.160063990834163</v>
       </c>
     </row>
     <row r="128">
@@ -20237,10 +19848,7 @@
         <v>-0.8899897505978819</v>
       </c>
       <c r="AZ128" t="n">
-        <v>0.3483273407058165</v>
-      </c>
-      <c r="BA128" t="n">
-        <v>14.95178371289261</v>
+        <v>3.483273407058165</v>
       </c>
     </row>
     <row r="129">
@@ -20406,10 +20014,7 @@
         <v>-0.9594183293878932</v>
       </c>
       <c r="AZ129" t="n">
-        <v>0.3335399262952408</v>
-      </c>
-      <c r="BA129" t="n">
-        <v>13.39656411771</v>
+        <v>3.335399262952408</v>
       </c>
     </row>
     <row r="130">
@@ -20575,10 +20180,7 @@
         <v>-0.8095535435529191</v>
       </c>
       <c r="AZ130" t="n">
-        <v>0.2816077793273518</v>
-      </c>
-      <c r="BA130" t="n">
-        <v>15.24780589347843</v>
+        <v>2.816077793273518</v>
       </c>
     </row>
     <row r="131">
@@ -20744,10 +20346,7 @@
         <v>-0.8061192631907587</v>
       </c>
       <c r="AZ131" t="n">
-        <v>0.2283823895902871</v>
-      </c>
-      <c r="BA131" t="n">
-        <v>12.36588830848125</v>
+        <v>2.283823895902871</v>
       </c>
     </row>
     <row r="132">
@@ -20913,10 +20512,7 @@
         <v>-0.9432647644326476</v>
       </c>
       <c r="AZ132" t="n">
-        <v>0.4425021074703185</v>
-      </c>
-      <c r="BA132" t="n">
-        <v>15.32398352756091</v>
+        <v>4.425021074703185</v>
       </c>
     </row>
     <row r="133">
@@ -21082,10 +20678,7 @@
         <v>-0.9047947568126941</v>
       </c>
       <c r="AZ133" t="n">
-        <v>0.3424239972728017</v>
-      </c>
-      <c r="BA133" t="n">
-        <v>15.37482698512445</v>
+        <v>3.424239972728016</v>
       </c>
     </row>
     <row r="134">
@@ -21251,10 +20844,7 @@
         <v>-0.925575101488498</v>
       </c>
       <c r="AZ134" t="n">
-        <v>0.2877727947098655</v>
-      </c>
-      <c r="BA134" t="n">
-        <v>12.64306724710941</v>
+        <v>2.877727947098654</v>
       </c>
     </row>
     <row r="135">
@@ -21420,10 +21010,7 @@
         <v>-0.8729547641963427</v>
       </c>
       <c r="AZ135" t="n">
-        <v>0.2286543990281047</v>
-      </c>
-      <c r="BA135" t="n">
-        <v>14.34571921902312</v>
+        <v>2.286543990281047</v>
       </c>
     </row>
     <row r="136">
@@ -21589,10 +21176,7 @@
         <v>-0.8111718275652702</v>
       </c>
       <c r="AZ136" t="n">
-        <v>0.212522899192218</v>
-      </c>
-      <c r="BA136" t="n">
-        <v>12.07681251870081</v>
+        <v>2.12522899192218</v>
       </c>
     </row>
     <row r="137">
@@ -21758,10 +21342,7 @@
         <v>-0.9191253037139883</v>
       </c>
       <c r="AZ137" t="n">
-        <v>0.2487492359828174</v>
-      </c>
-      <c r="BA137" t="n">
-        <v>12.92788698041661</v>
+        <v>2.487492359828174</v>
       </c>
     </row>
     <row r="138">
@@ -21927,10 +21508,7 @@
         <v>-0.983991462113127</v>
       </c>
       <c r="AZ138" t="n">
-        <v>0.3634267201648407</v>
-      </c>
-      <c r="BA138" t="n">
-        <v>12.61555674855043</v>
+        <v>3.634267201648408</v>
       </c>
     </row>
     <row r="139">
@@ -21975,7 +21553,7 @@
         <v>-30.32987330795573</v>
       </c>
       <c r="K139" t="n">
-        <v>0.02957614146330922</v>
+        <v>0.0117556</v>
       </c>
       <c r="L139" t="n">
         <v>2.373333643299183</v>
@@ -22090,16 +21668,13 @@
         <v>0.5165860400829302</v>
       </c>
       <c r="AX139" t="n">
-        <v>16.82978356315537</v>
+        <v>42.34237805477897</v>
       </c>
       <c r="AY139" t="n">
         <v>-0.8676616915422886</v>
       </c>
       <c r="AZ139" t="n">
-        <v>0.887896060770315</v>
-      </c>
-      <c r="BA139" t="n">
-        <v>14.94309852934265</v>
+        <v>3.529111782529205</v>
       </c>
     </row>
     <row r="140">
@@ -22265,10 +21840,7 @@
         <v>-0.9794520547945206</v>
       </c>
       <c r="AZ140" t="n">
-        <v>0.2763025421902743</v>
-      </c>
-      <c r="BA140" t="n">
-        <v>13.50197279742473</v>
+        <v>2.763025421902743</v>
       </c>
     </row>
     <row r="141">
@@ -22434,10 +22006,7 @@
         <v>-0.8755935422602089</v>
       </c>
       <c r="AZ141" t="n">
-        <v>0.3071371534917146</v>
-      </c>
-      <c r="BA141" t="n">
-        <v>14.89304857028718</v>
+        <v>3.071371534917147</v>
       </c>
     </row>
     <row r="142">
@@ -22603,10 +22172,7 @@
         <v>-0.8558154437680231</v>
       </c>
       <c r="AZ142" t="n">
-        <v>0.2351665444744986</v>
-      </c>
-      <c r="BA142" t="n">
-        <v>12.33569292798704</v>
+        <v>2.351665444744986</v>
       </c>
     </row>
     <row r="143">
@@ -22772,10 +22338,7 @@
         <v>-0.910299003322259</v>
       </c>
       <c r="AZ143" t="n">
-        <v>0.2634069568539765</v>
-      </c>
-      <c r="BA143" t="n">
-        <v>13.20241292636161</v>
+        <v>2.634069568539765</v>
       </c>
     </row>
     <row r="144">
@@ -22941,10 +22504,7 @@
         <v>-0.8479307025986524</v>
       </c>
       <c r="AZ144" t="n">
-        <v>0.2850083474322018</v>
-      </c>
-      <c r="BA144" t="n">
-        <v>14.72041205661443</v>
+        <v>2.850083474322018</v>
       </c>
     </row>
     <row r="145">
@@ -23110,10 +22670,7 @@
         <v>-0.9031939413895291</v>
       </c>
       <c r="AZ145" t="n">
-        <v>0.3306302943724049</v>
-      </c>
-      <c r="BA145" t="n">
-        <v>13.50483650630982</v>
+        <v>3.306302943724048</v>
       </c>
     </row>
     <row r="146">
@@ -23279,10 +22836,7 @@
         <v>-0.8867924528301887</v>
       </c>
       <c r="AZ146" t="n">
-        <v>0.3753925003975221</v>
-      </c>
-      <c r="BA146" t="n">
-        <v>14.04704424717668</v>
+        <v>3.753925003975221</v>
       </c>
     </row>
     <row r="147">
@@ -23448,10 +23002,7 @@
         <v>-0.9927797833935018</v>
       </c>
       <c r="AZ147" t="n">
-        <v>0.275498874631122</v>
-      </c>
-      <c r="BA147" t="n">
-        <v>12.39357609552841</v>
+        <v>2.754988746311219</v>
       </c>
     </row>
     <row r="148">
@@ -23617,10 +23168,7 @@
         <v>-0.8752424046541692</v>
       </c>
       <c r="AZ148" t="n">
-        <v>0.204352754630459</v>
-      </c>
-      <c r="BA148" t="n">
-        <v>12.73705359648974</v>
+        <v>2.043527546304591</v>
       </c>
     </row>
     <row r="149">
@@ -23786,10 +23334,7 @@
         <v>-0.9457209457209457</v>
       </c>
       <c r="AZ149" t="n">
-        <v>0.1613708822578354</v>
-      </c>
-      <c r="BA149" t="n">
-        <v>10.17299216629021</v>
+        <v>1.613708822578354</v>
       </c>
     </row>
     <row r="150">
@@ -23955,10 +23500,7 @@
         <v>-0.8900032351989647</v>
       </c>
       <c r="AZ150" t="n">
-        <v>0.2776338886342699</v>
-      </c>
-      <c r="BA150" t="n">
-        <v>15.42719268663395</v>
+        <v>2.776338886342698</v>
       </c>
     </row>
     <row r="151">
@@ -24124,10 +23666,7 @@
         <v>-0.9144542772861356</v>
       </c>
       <c r="AZ151" t="n">
-        <v>0.1992943083149607</v>
-      </c>
-      <c r="BA151" t="n">
-        <v>12.29805279278685</v>
+        <v>1.992943083149608</v>
       </c>
     </row>
     <row r="152">
@@ -24293,10 +23832,7 @@
         <v>-0.870988867059594</v>
       </c>
       <c r="AZ152" t="n">
-        <v>0.2929222953305048</v>
-      </c>
-      <c r="BA152" t="n">
-        <v>13.84738554555246</v>
+        <v>2.929222953305048</v>
       </c>
     </row>
     <row r="153">
@@ -24462,10 +23998,7 @@
         <v>-0.9734422880490295</v>
       </c>
       <c r="AZ153" t="n">
-        <v>0.278928268195533</v>
-      </c>
-      <c r="BA153" t="n">
-        <v>12.99811599897735</v>
+        <v>2.78928268195533</v>
       </c>
     </row>
     <row r="154">
@@ -24631,10 +24164,7 @@
         <v>-0.8216748768472907</v>
       </c>
       <c r="AZ154" t="n">
-        <v>0.3594130595075935</v>
-      </c>
-      <c r="BA154" t="n">
-        <v>13.08294443919041</v>
+        <v>3.594130595075935</v>
       </c>
     </row>
     <row r="155">
@@ -24800,10 +24330,7 @@
         <v>-0.8612735542560104</v>
       </c>
       <c r="AZ155" t="n">
-        <v>0.2320891755316213</v>
-      </c>
-      <c r="BA155" t="n">
-        <v>12.9060602060763</v>
+        <v>2.320891755316213</v>
       </c>
     </row>
     <row r="156">
@@ -24969,10 +24496,7 @@
         <v>-1.018099547511312</v>
       </c>
       <c r="AZ156" t="n">
-        <v>0.3462797777914783</v>
-      </c>
-      <c r="BA156" t="n">
-        <v>14.93215294918606</v>
+        <v>3.462797777914784</v>
       </c>
     </row>
     <row r="157">
@@ -25138,10 +24662,7 @@
         <v>-1.04876299749014</v>
       </c>
       <c r="AZ157" t="n">
-        <v>0.3554401383644461</v>
-      </c>
-      <c r="BA157" t="n">
-        <v>15.32716274738345</v>
+        <v>3.554401383644462</v>
       </c>
     </row>
     <row r="158">
@@ -25307,10 +24828,7 @@
         <v>-0.8695652173913042</v>
       </c>
       <c r="AZ158" t="n">
-        <v>0.3274162961093018</v>
-      </c>
-      <c r="BA158" t="n">
-        <v>13.30667483923764</v>
+        <v>3.274162961093018</v>
       </c>
     </row>
     <row r="159">
@@ -25472,10 +24990,7 @@
       </c>
       <c r="AY159" t="inlineStr"/>
       <c r="AZ159" t="n">
-        <v>0.3352256061133059</v>
-      </c>
-      <c r="BA159" t="n">
-        <v>13.36339572806621</v>
+        <v>3.352256061133059</v>
       </c>
     </row>
     <row r="160">
@@ -25637,10 +25152,7 @@
       </c>
       <c r="AY160" t="inlineStr"/>
       <c r="AZ160" t="n">
-        <v>0.2434472726667247</v>
-      </c>
-      <c r="BA160" t="n">
-        <v>12.29154143560339</v>
+        <v>2.434472726667246</v>
       </c>
     </row>
     <row r="161">
@@ -25806,10 +25318,7 @@
         <v>-0.9148648648648647</v>
       </c>
       <c r="AZ161" t="n">
-        <v>0.2193729066609965</v>
-      </c>
-      <c r="BA161" t="n">
-        <v>11.64590440849937</v>
+        <v>2.193729066609965</v>
       </c>
     </row>
     <row r="162">
@@ -25975,10 +25484,7 @@
         <v>-0.875</v>
       </c>
       <c r="AZ162" t="n">
-        <v>0.2693134402703707</v>
-      </c>
-      <c r="BA162" t="n">
-        <v>12.17300558723502</v>
+        <v>2.693134402703707</v>
       </c>
     </row>
     <row r="163">
@@ -26144,10 +25650,7 @@
         <v>-0.9019350606756315</v>
       </c>
       <c r="AZ163" t="n">
-        <v>0.2786500146224659</v>
-      </c>
-      <c r="BA163" t="n">
-        <v>13.42169439208957</v>
+        <v>2.786500146224659</v>
       </c>
     </row>
     <row r="164">
@@ -26313,10 +25816,7 @@
         <v>-0.8602257636122178</v>
       </c>
       <c r="AZ164" t="n">
-        <v>0.3302696303234725</v>
-      </c>
-      <c r="BA164" t="n">
-        <v>14.07419437917497</v>
+        <v>3.302696303234725</v>
       </c>
     </row>
     <row r="165">
@@ -26482,10 +25982,7 @@
         <v>-0.8340425531914893</v>
       </c>
       <c r="AZ165" t="n">
-        <v>0.3140509103601919</v>
-      </c>
-      <c r="BA165" t="n">
-        <v>13.33772096173453</v>
+        <v>3.140509103601919</v>
       </c>
     </row>
     <row r="166">
@@ -26651,10 +26148,7 @@
         <v>-0.9123961218836566</v>
       </c>
       <c r="AZ166" t="n">
-        <v>0.4419867263324095</v>
-      </c>
-      <c r="BA166" t="n">
-        <v>16.97539046167085</v>
+        <v>4.419867263324095</v>
       </c>
     </row>
     <row r="167">
@@ -26820,10 +26314,7 @@
         <v>-0.9287135278514589</v>
       </c>
       <c r="AZ167" t="n">
-        <v>0.2822534280040117</v>
-      </c>
-      <c r="BA167" t="n">
-        <v>11.65132875248652</v>
+        <v>2.822534280040117</v>
       </c>
     </row>
     <row r="168">
@@ -26989,10 +26480,7 @@
         <v>-0.794580970384373</v>
       </c>
       <c r="AZ168" t="n">
-        <v>0.3720589980627997</v>
-      </c>
-      <c r="BA168" t="n">
-        <v>15.11954301763624</v>
+        <v>3.720589980627997</v>
       </c>
     </row>
     <row r="169">
@@ -27158,10 +26646,7 @@
         <v>-0.8666886109282422</v>
       </c>
       <c r="AZ169" t="n">
-        <v>0.3370510290002701</v>
-      </c>
-      <c r="BA169" t="n">
-        <v>12.83721020627359</v>
+        <v>3.370510290002701</v>
       </c>
     </row>
     <row r="170">
@@ -27327,10 +26812,7 @@
         <v>-0.8734652114597544</v>
       </c>
       <c r="AZ170" t="n">
-        <v>0.3618600999053327</v>
-      </c>
-      <c r="BA170" t="n">
-        <v>15.67979022827618</v>
+        <v>3.618600999053328</v>
       </c>
     </row>
     <row r="171">
@@ -27496,10 +26978,7 @@
         <v>-0.9163306451612903</v>
       </c>
       <c r="AZ171" t="n">
-        <v>0.254785183807967</v>
-      </c>
-      <c r="BA171" t="n">
-        <v>11.61765076524852</v>
+        <v>2.547851838079669</v>
       </c>
     </row>
     <row r="172">
@@ -27665,10 +27144,7 @@
         <v>-0.8450749123366273</v>
       </c>
       <c r="AZ172" t="n">
-        <v>0.3188696860136649</v>
-      </c>
-      <c r="BA172" t="n">
-        <v>14.69626650381366</v>
+        <v>3.18869686013665</v>
       </c>
     </row>
     <row r="173">
@@ -27834,10 +27310,7 @@
         <v>-0.8522613065326633</v>
       </c>
       <c r="AZ173" t="n">
-        <v>0.399707243754127</v>
-      </c>
-      <c r="BA173" t="n">
-        <v>12.47173871860493</v>
+        <v>3.99707243754127</v>
       </c>
     </row>
     <row r="174">
@@ -28003,10 +27476,7 @@
         <v>-0.9190476190476191</v>
       </c>
       <c r="AZ174" t="n">
-        <v>0.3801718619146223</v>
-      </c>
-      <c r="BA174" t="n">
-        <v>14.2475185393632</v>
+        <v>3.801718619146223</v>
       </c>
     </row>
     <row r="175">
@@ -28172,10 +27642,7 @@
         <v>-0.8253346392425727</v>
       </c>
       <c r="AZ175" t="n">
-        <v>0.2470312536106503</v>
-      </c>
-      <c r="BA175" t="n">
-        <v>11.3388765448196</v>
+        <v>2.470312536106503</v>
       </c>
     </row>
     <row r="176">
@@ -28341,10 +27808,7 @@
         <v>-0.8593242365172189</v>
       </c>
       <c r="AZ176" t="n">
-        <v>0.2303895675632164</v>
-      </c>
-      <c r="BA176" t="n">
-        <v>10.92082410889718</v>
+        <v>2.303895675632163</v>
       </c>
     </row>
     <row r="177">
@@ -28510,10 +27974,7 @@
         <v>-1.011280931586608</v>
       </c>
       <c r="AZ177" t="n">
-        <v>0.2939442645614514</v>
-      </c>
-      <c r="BA177" t="n">
-        <v>13.1516753899925</v>
+        <v>2.939442645614514</v>
       </c>
     </row>
     <row r="178">
@@ -28679,10 +28140,7 @@
         <v>-0.8638230647709321</v>
       </c>
       <c r="AZ178" t="n">
-        <v>0.3054467120359153</v>
-      </c>
-      <c r="BA178" t="n">
-        <v>13.45013914035445</v>
+        <v>3.054467120359153</v>
       </c>
     </row>
     <row r="179">
@@ -28848,10 +28306,7 @@
         <v>-0.8194444444444445</v>
       </c>
       <c r="AZ179" t="n">
-        <v>0.2464363334952325</v>
-      </c>
-      <c r="BA179" t="n">
-        <v>13.35702874314139</v>
+        <v>2.464363334952325</v>
       </c>
     </row>
     <row r="180">
@@ -29017,10 +28472,7 @@
         <v>-0.8907371167645139</v>
       </c>
       <c r="AZ180" t="n">
-        <v>0.3280651598232026</v>
-      </c>
-      <c r="BA180" t="n">
-        <v>12.92183174935129</v>
+        <v>3.280651598232026</v>
       </c>
     </row>
     <row r="181">
@@ -29186,10 +28638,7 @@
         <v>-0.9359058207979072</v>
       </c>
       <c r="AZ181" t="n">
-        <v>0.3562090494563998</v>
-      </c>
-      <c r="BA181" t="n">
-        <v>15.23965851812918</v>
+        <v>3.562090494563997</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update R ahora en Cleaning
</commit_message>
<xml_diff>
--- a/Results_isofys/Numex_preliminar_base.xlsx
+++ b/Results_isofys/Numex_preliminar_base.xlsx
@@ -904,13 +904,13 @@
         <v>0.586048687666667</v>
       </c>
       <c r="BE2" t="n">
-        <v>1583.411527786951</v>
+        <v>1.583411527786951</v>
       </c>
       <c r="BF2" t="n">
-        <v>62678.6295709413</v>
+        <v>62.6786295709413</v>
       </c>
       <c r="BG2" t="n">
-        <v>81.98919152048342</v>
+        <v>0.08198919152048342</v>
       </c>
       <c r="BH2" t="n">
         <v>764.4742972649296</v>
@@ -1089,13 +1089,13 @@
         <v>0.827745731739708</v>
       </c>
       <c r="BE3" t="n">
-        <v>1927.929018543231</v>
+        <v>1.927929018543231</v>
       </c>
       <c r="BF3" t="n">
-        <v>49313.98966307422</v>
+        <v>49.31398966307422</v>
       </c>
       <c r="BG3" t="n">
-        <v>85.97204781478952</v>
+        <v>0.08597204781478951</v>
       </c>
       <c r="BH3" t="n">
         <v>573.6049206285264</v>
@@ -1274,13 +1274,13 @@
         <v>0.586801039508632</v>
       </c>
       <c r="BE4" t="n">
-        <v>1459.443363957555</v>
+        <v>1.459443363957555</v>
       </c>
       <c r="BF4" t="n">
-        <v>62014.10491775165</v>
+        <v>62.01410491775165</v>
       </c>
       <c r="BG4" t="n">
-        <v>80.23105743376664</v>
+        <v>0.08023105743376663</v>
       </c>
       <c r="BH4" t="n">
         <v>772.9438811017334</v>
@@ -1459,13 +1459,13 @@
         <v>0.7090190245683931</v>
       </c>
       <c r="BE5" t="n">
-        <v>2308.390026071944</v>
+        <v>2.308390026071944</v>
       </c>
       <c r="BF5" t="n">
-        <v>68039.66990152447</v>
+        <v>68.03966990152448</v>
       </c>
       <c r="BG5" t="n">
-        <v>102.5630023455334</v>
+        <v>0.1025630023455334</v>
       </c>
       <c r="BH5" t="n">
         <v>663.3938978531428</v>
@@ -1644,13 +1644,13 @@
         <v>0.629324291421087</v>
       </c>
       <c r="BE6" t="n">
-        <v>1972.952651382424</v>
+        <v>1.972952651382424</v>
       </c>
       <c r="BF6" t="n">
-        <v>58140.10355624786</v>
+        <v>58.14010355624787</v>
       </c>
       <c r="BG6" t="n">
-        <v>76.36880331298339</v>
+        <v>0.07636880331298337</v>
       </c>
       <c r="BH6" t="n">
         <v>761.3069870686782</v>
@@ -1829,13 +1829,13 @@
         <v>0.85184102744709</v>
       </c>
       <c r="BE7" t="n">
-        <v>2411.024955423218</v>
+        <v>2.411024955423218</v>
       </c>
       <c r="BF7" t="n">
-        <v>63936.67365779264</v>
+        <v>63.93667365779265</v>
       </c>
       <c r="BG7" t="n">
-        <v>125.6379244892002</v>
+        <v>0.1256379244892002</v>
       </c>
       <c r="BH7" t="n">
         <v>508.8962900154292</v>
@@ -2014,13 +2014,13 @@
         <v>0.666581855706874</v>
       </c>
       <c r="BE8" t="n">
-        <v>2212.734935521185</v>
+        <v>2.212734935521185</v>
       </c>
       <c r="BF8" t="n">
-        <v>65829.19875238115</v>
+        <v>65.82919875238116</v>
       </c>
       <c r="BG8" t="n">
-        <v>92.64851857109888</v>
+        <v>0.09264851857109888</v>
       </c>
       <c r="BH8" t="n">
         <v>710.5261883044957</v>
@@ -2199,13 +2199,13 @@
         <v>0.525173295666667</v>
       </c>
       <c r="BE9" t="n">
-        <v>2491.330280495736</v>
+        <v>2.491330280495736</v>
       </c>
       <c r="BF9" t="n">
-        <v>70465.3963916366</v>
+        <v>70.4653963916366</v>
       </c>
       <c r="BG9" t="n">
-        <v>75.68407956598034</v>
+        <v>0.07568407956598033</v>
       </c>
       <c r="BH9" t="n">
         <v>931.0464868665787</v>
@@ -2384,13 +2384,13 @@
         <v>0.907511655978624</v>
       </c>
       <c r="BE10" t="n">
-        <v>1922.442143630735</v>
+        <v>1.922442143630735</v>
       </c>
       <c r="BF10" t="n">
-        <v>53859.76820401974</v>
+        <v>53.85976820401974</v>
       </c>
       <c r="BG10" t="n">
-        <v>101.7744649299599</v>
+        <v>0.1017744649299599</v>
       </c>
       <c r="BH10" t="n">
         <v>529.2070878592726</v>
@@ -2569,13 +2569,13 @@
         <v>0.578893611326861</v>
       </c>
       <c r="BE11" t="n">
-        <v>1541.538771183675</v>
+        <v>1.541538771183675</v>
       </c>
       <c r="BF11" t="n">
-        <v>61569.64889603419</v>
+        <v>61.56964889603419</v>
       </c>
       <c r="BG11" t="n">
-        <v>80.19603864765268</v>
+        <v>0.08019603864765268</v>
       </c>
       <c r="BH11" t="n">
         <v>767.7392790751805</v>
@@ -2754,13 +2754,13 @@
         <v>0.627050194054776</v>
       </c>
       <c r="BE12" t="n">
-        <v>1704.503359635594</v>
+        <v>1.704503359635594</v>
       </c>
       <c r="BF12" t="n">
-        <v>70453.9122144526</v>
+        <v>70.4539122144526</v>
       </c>
       <c r="BG12" t="n">
-        <v>96.68356330223143</v>
+        <v>0.09668356330223143</v>
       </c>
       <c r="BH12" t="n">
         <v>728.7062020481669</v>
@@ -2939,13 +2939,13 @@
         <v>1.21053150264026</v>
       </c>
       <c r="BE13" t="n">
-        <v>1893.086604314296</v>
+        <v>1.893086604314296</v>
       </c>
       <c r="BF13" t="n">
-        <v>62982.27944361334</v>
+        <v>62.98227944361334</v>
       </c>
       <c r="BG13" t="n">
-        <v>169.6420166821183</v>
+        <v>0.1696420166821183</v>
       </c>
       <c r="BH13" t="n">
         <v>371.265802396301</v>
@@ -3124,13 +3124,13 @@
         <v>2.15640457208089</v>
       </c>
       <c r="BE14" t="n">
-        <v>2420.263723581012</v>
+        <v>2.420263723581012</v>
       </c>
       <c r="BF14" t="n">
-        <v>59335.47349313596</v>
+        <v>59.33547349313596</v>
       </c>
       <c r="BG14" t="n">
-        <v>290.6871507126771</v>
+        <v>0.2906871507126771</v>
       </c>
       <c r="BH14" t="n">
         <v>204.1214183277908</v>
@@ -3309,13 +3309,13 @@
         <v>0.8031287501650169</v>
       </c>
       <c r="BE15" t="n">
-        <v>2262.696828216982</v>
+        <v>2.262696828216982</v>
       </c>
       <c r="BF15" t="n">
-        <v>67377.42901484933</v>
+        <v>67.37742901484933</v>
       </c>
       <c r="BG15" t="n">
-        <v>113.1241952885253</v>
+        <v>0.1131241952885253</v>
       </c>
       <c r="BH15" t="n">
         <v>595.6058192767865</v>
@@ -3494,13 +3494,13 @@
         <v>0.543376352145214</v>
       </c>
       <c r="BE16" t="n">
-        <v>2346.594974817986</v>
+        <v>2.346594974817986</v>
       </c>
       <c r="BF16" t="n">
-        <v>75854.79688556591</v>
+        <v>75.85479688556592</v>
       </c>
       <c r="BG16" t="n">
-        <v>86.60033209198477</v>
+        <v>0.08660033209198477</v>
       </c>
       <c r="BH16" t="n">
         <v>875.9180831430851</v>
@@ -3679,13 +3679,13 @@
         <v>0.614479672666667</v>
       </c>
       <c r="BE17" t="n">
-        <v>2040.293659175826</v>
+        <v>2.040293659175827</v>
       </c>
       <c r="BF17" t="n">
-        <v>57933.09073325802</v>
+        <v>57.93309073325802</v>
       </c>
       <c r="BG17" t="n">
-        <v>73.8952274288045</v>
+        <v>0.0738952274288045</v>
       </c>
       <c r="BH17" t="n">
         <v>783.9896127131425</v>
@@ -3864,13 +3864,13 @@
         <v>0.733080008530184</v>
       </c>
       <c r="BE18" t="n">
-        <v>2199.748552043699</v>
+        <v>2.199748552043698</v>
       </c>
       <c r="BF18" t="n">
-        <v>64181.04834646514</v>
+        <v>64.18104834646515</v>
       </c>
       <c r="BG18" t="n">
-        <v>97.23724315459992</v>
+        <v>0.09723724315459993</v>
       </c>
       <c r="BH18" t="n">
         <v>660.0459480779612</v>
@@ -4049,13 +4049,13 @@
         <v>0.692635240264026</v>
       </c>
       <c r="BE19" t="n">
-        <v>1804.095984933663</v>
+        <v>1.804095984933663</v>
       </c>
       <c r="BF19" t="n">
-        <v>48111.20672929789</v>
+        <v>48.11120672929789</v>
       </c>
       <c r="BG19" t="n">
-        <v>71.36813755565903</v>
+        <v>0.07136813755565903</v>
       </c>
       <c r="BH19" t="n">
         <v>674.1272559029107</v>
@@ -4234,13 +4234,13 @@
         <v>0.549719054790026</v>
       </c>
       <c r="BE20" t="n">
-        <v>2216.436966512492</v>
+        <v>2.216436966512492</v>
       </c>
       <c r="BF20" t="n">
-        <v>68165.10648324604</v>
+        <v>68.16510648324603</v>
       </c>
       <c r="BG20" t="n">
-        <v>76.53916563813738</v>
+        <v>0.07653916563813738</v>
       </c>
       <c r="BH20" t="n">
         <v>890.5911883795245</v>
@@ -4419,13 +4419,13 @@
         <v>1.16688620768229</v>
       </c>
       <c r="BE21" t="n">
-        <v>2731.252805030631</v>
+        <v>2.731252805030631</v>
       </c>
       <c r="BF21" t="n">
-        <v>62693.41168086865</v>
+        <v>62.69341168086865</v>
       </c>
       <c r="BG21" t="n">
-        <v>167.791336712078</v>
+        <v>0.1677913367120781</v>
       </c>
       <c r="BH21" t="n">
         <v>373.6391455564095</v>
@@ -4604,13 +4604,13 @@
         <v>0.472759833658854</v>
       </c>
       <c r="BE22" t="n">
-        <v>1359.691165823957</v>
+        <v>1.359691165823957</v>
       </c>
       <c r="BF22" t="n">
-        <v>72098.69586996443</v>
+        <v>72.09869586996444</v>
       </c>
       <c r="BG22" t="n">
-        <v>78.81098756214665</v>
+        <v>0.07881098756214665</v>
       </c>
       <c r="BH22" t="n">
         <v>914.8305090468607</v>
@@ -4789,13 +4789,13 @@
         <v>0.541857143239625</v>
       </c>
       <c r="BE23" t="n">
-        <v>1532.285064088778</v>
+        <v>1.532285064088778</v>
       </c>
       <c r="BF23" t="n">
-        <v>58814.77292575601</v>
+        <v>58.814772925756</v>
       </c>
       <c r="BG23" t="n">
-        <v>72.14665247249056</v>
+        <v>0.07214665247249055</v>
       </c>
       <c r="BH23" t="n">
         <v>815.2113911062197</v>
@@ -4974,13 +4974,13 @@
         <v>0.907596492739274</v>
       </c>
       <c r="BE24" t="n">
-        <v>2083.919474390169</v>
+        <v>2.083919474390169</v>
       </c>
       <c r="BF24" t="n">
-        <v>64502.69324889292</v>
+        <v>64.50269324889292</v>
       </c>
       <c r="BG24" t="n">
-        <v>133.6534991978402</v>
+        <v>0.1336534991978402</v>
       </c>
       <c r="BH24" t="n">
         <v>482.6113318096744</v>
@@ -5159,13 +5159,13 @@
         <v>0.689000921175685</v>
       </c>
       <c r="BE25" t="n">
-        <v>1924.962019984864</v>
+        <v>1.924962019984864</v>
       </c>
       <c r="BF25" t="n">
-        <v>59226.28309595306</v>
+        <v>59.22628309595306</v>
       </c>
       <c r="BG25" t="n">
-        <v>84.04879803272316</v>
+        <v>0.08404879803272315</v>
       </c>
       <c r="BH25" t="n">
         <v>704.6654382004866</v>
@@ -5344,13 +5344,13 @@
         <v>0.702029613176778</v>
       </c>
       <c r="BE26" t="n">
-        <v>1993.680458705612</v>
+        <v>1.993680458705612</v>
       </c>
       <c r="BF26" t="n">
-        <v>58198.73982352419</v>
+        <v>58.19873982352419</v>
       </c>
       <c r="BG26" t="n">
-        <v>86.06477042797445</v>
+        <v>0.08606477042797446</v>
       </c>
       <c r="BH26" t="n">
         <v>676.2202412685143</v>
@@ -5529,13 +5529,13 @@
         <v>1.17576645368558</v>
       </c>
       <c r="BE27" t="n">
-        <v>2247.906864753312</v>
+        <v>2.247906864753312</v>
       </c>
       <c r="BF27" t="n">
-        <v>43536.30630525455</v>
+        <v>43.53630630525455</v>
       </c>
       <c r="BG27" t="n">
-        <v>115.5297984473839</v>
+        <v>0.1155297984473839</v>
       </c>
       <c r="BH27" t="n">
         <v>376.8404938842028</v>
@@ -5714,13 +5714,13 @@
         <v>2.73427812416332</v>
       </c>
       <c r="BE28" t="n">
-        <v>1941.969337398241</v>
+        <v>1.941969337398241</v>
       </c>
       <c r="BF28" t="n">
-        <v>61803.18961158281</v>
+        <v>61.80318961158282</v>
       </c>
       <c r="BG28" t="n">
-        <v>392.4651391362423</v>
+        <v>0.3924651391362423</v>
       </c>
       <c r="BH28" t="n">
         <v>157.4743421736833</v>
@@ -5899,13 +5899,13 @@
         <v>1.40558051353135</v>
       </c>
       <c r="BE29" t="n">
-        <v>2299.853817964811</v>
+        <v>2.299853817964811</v>
       </c>
       <c r="BF29" t="n">
-        <v>47703.9521233669</v>
+        <v>47.7039521233669</v>
       </c>
       <c r="BG29" t="n">
-        <v>148.4202958654755</v>
+        <v>0.1484202958654755</v>
       </c>
       <c r="BH29" t="n">
         <v>321.4112453097694</v>
@@ -6084,13 +6084,13 @@
         <v>0.840966547043011</v>
       </c>
       <c r="BE30" t="n">
-        <v>2056.480718564838</v>
+        <v>2.056480718564838</v>
       </c>
       <c r="BF30" t="n">
-        <v>60032.56549989229</v>
+        <v>60.03256549989229</v>
       </c>
       <c r="BG30" t="n">
-        <v>106.5298553812398</v>
+        <v>0.1065298553812398</v>
       </c>
       <c r="BH30" t="n">
         <v>563.528085953491</v>
@@ -6269,13 +6269,13 @@
         <v>1.68222301339869</v>
       </c>
       <c r="BE31" t="n">
-        <v>1366.31885562437</v>
+        <v>1.36631885562437</v>
       </c>
       <c r="BF31" t="n">
-        <v>58714.22404388255</v>
+        <v>58.71422404388255</v>
       </c>
       <c r="BG31" t="n">
-        <v>230.0974793772151</v>
+        <v>0.2300974793772151</v>
       </c>
       <c r="BH31" t="n">
         <v>255.1710875008246</v>
@@ -6454,13 +6454,13 @@
         <v>1.12802003685584</v>
       </c>
       <c r="BE32" t="n">
-        <v>2060.536274187499</v>
+        <v>2.060536274187499</v>
       </c>
       <c r="BF32" t="n">
-        <v>42488.72527334292</v>
+        <v>42.48872527334292</v>
       </c>
       <c r="BG32" t="n">
-        <v>107.993509188816</v>
+        <v>0.107993509188816</v>
       </c>
       <c r="BH32" t="n">
         <v>393.437768551956</v>
@@ -6639,13 +6639,13 @@
         <v>1.00512667963684</v>
       </c>
       <c r="BE33" t="n">
-        <v>2140.487849336566</v>
+        <v>2.140487849336566</v>
       </c>
       <c r="BF33" t="n">
-        <v>47071.79999838402</v>
+        <v>47.07179999838402</v>
       </c>
       <c r="BG33" t="n">
-        <v>112.1486530696386</v>
+        <v>0.1121486530696386</v>
       </c>
       <c r="BH33" t="n">
         <v>419.7268420972906</v>
@@ -6824,13 +6824,13 @@
         <v>2.08665858366667</v>
       </c>
       <c r="BE34" t="n">
-        <v>1262.484116656831</v>
+        <v>1.262484116656831</v>
       </c>
       <c r="BF34" t="n">
-        <v>55387.52547725021</v>
+        <v>55.38752547725021</v>
       </c>
       <c r="BG34" t="n">
-        <v>261.6555036990323</v>
+        <v>0.2616555036990323</v>
       </c>
       <c r="BH34" t="n">
         <v>211.6811024199185</v>
@@ -7009,13 +7009,13 @@
         <v>0.774807667332003</v>
       </c>
       <c r="BE35" t="n">
-        <v>2368.53606683806</v>
+        <v>2.36853606683806</v>
       </c>
       <c r="BF35" t="n">
-        <v>57270.8070874746</v>
+        <v>57.27080708747459</v>
       </c>
       <c r="BG35" t="n">
-        <v>91.57430319646703</v>
+        <v>0.09157430319646703</v>
       </c>
       <c r="BH35" t="n">
         <v>625.4025975453355</v>
@@ -7194,13 +7194,13 @@
         <v>1.94216136813922</v>
       </c>
       <c r="BE36" t="n">
-        <v>1404.492354378129</v>
+        <v>1.404492354378129</v>
       </c>
       <c r="BF36" t="n">
-        <v>64215.80057406097</v>
+        <v>64.21580057406096</v>
       </c>
       <c r="BG36" t="n">
-        <v>287.9610376304444</v>
+        <v>0.2879610376304444</v>
       </c>
       <c r="BH36" t="n">
         <v>223.0016987800707</v>
@@ -7379,13 +7379,13 @@
         <v>0.628281845285525</v>
       </c>
       <c r="BE37" t="n">
-        <v>1657.36668134432</v>
+        <v>1.65736668134432</v>
       </c>
       <c r="BF37" t="n">
-        <v>53824.76778431748</v>
+        <v>53.82476778431748</v>
       </c>
       <c r="BG37" t="n">
-        <v>75.01750757791727</v>
+        <v>0.07501750757791728</v>
       </c>
       <c r="BH37" t="n">
         <v>717.496082210038</v>
@@ -7564,13 +7564,13 @@
         <v>0.750170432291667</v>
       </c>
       <c r="BE38" t="n">
-        <v>2537.0946862891</v>
+        <v>2.5370946862891</v>
       </c>
       <c r="BF38" t="n">
-        <v>79264.49640071606</v>
+        <v>79.26449640071606</v>
       </c>
       <c r="BG38" t="n">
-        <v>132.9760039281311</v>
+        <v>0.1329760039281311</v>
       </c>
       <c r="BH38" t="n">
         <v>596.0812030684556</v>
@@ -7749,13 +7749,13 @@
         <v>0.961635565666667</v>
       </c>
       <c r="BE39" t="n">
-        <v>1790.085898974969</v>
+        <v>1.790085898974969</v>
       </c>
       <c r="BF39" t="n">
-        <v>39902.34824028318</v>
+        <v>39.90234824028317</v>
       </c>
       <c r="BG39" t="n">
-        <v>85.81442940428201</v>
+        <v>0.08581442940428201</v>
       </c>
       <c r="BH39" t="n">
         <v>464.9841351539898</v>
@@ -7934,13 +7934,13 @@
         <v>0.672914162127108</v>
       </c>
       <c r="BE40" t="n">
-        <v>1636.334848571583</v>
+        <v>1.636334848571583</v>
       </c>
       <c r="BF40" t="n">
-        <v>67019.60533465813</v>
+        <v>67.01960533465812</v>
       </c>
       <c r="BG40" t="n">
-        <v>99.41332983713632</v>
+        <v>0.09941332983713633</v>
       </c>
       <c r="BH40" t="n">
         <v>674.1510966834412</v>
@@ -8119,13 +8119,13 @@
         <v>0.631807111000663</v>
       </c>
       <c r="BE41" t="n">
-        <v>1962.293560349081</v>
+        <v>1.962293560349081</v>
       </c>
       <c r="BF41" t="n">
-        <v>64069.93482654983</v>
+        <v>64.06993482654983</v>
       </c>
       <c r="BG41" t="n">
-        <v>84.18811911277291</v>
+        <v>0.08418811911277291</v>
       </c>
       <c r="BH41" t="n">
         <v>761.0329759324582</v>
@@ -8304,13 +8304,13 @@
         <v>0.631807111000663</v>
       </c>
       <c r="BE42" t="n">
-        <v>1962.293560349081</v>
+        <v>1.962293560349081</v>
       </c>
       <c r="BF42" t="n">
-        <v>64069.93482654983</v>
+        <v>64.06993482654983</v>
       </c>
       <c r="BG42" t="n">
-        <v>84.18811911277291</v>
+        <v>0.08418811911277291</v>
       </c>
       <c r="BH42" t="n">
         <v>761.0329759324582</v>
@@ -8489,13 +8489,13 @@
         <v>0.631807111000663</v>
       </c>
       <c r="BE43" t="n">
-        <v>1962.293560349081</v>
+        <v>1.962293560349081</v>
       </c>
       <c r="BF43" t="n">
-        <v>64069.93482654983</v>
+        <v>64.06993482654983</v>
       </c>
       <c r="BG43" t="n">
-        <v>84.18811911277291</v>
+        <v>0.08418811911277291</v>
       </c>
       <c r="BH43" t="n">
         <v>761.0329759324582</v>
@@ -8674,13 +8674,13 @@
         <v>0.631807111000663</v>
       </c>
       <c r="BE44" t="n">
-        <v>1962.293560349081</v>
+        <v>1.962293560349081</v>
       </c>
       <c r="BF44" t="n">
-        <v>64069.93482654983</v>
+        <v>64.06993482654983</v>
       </c>
       <c r="BG44" t="n">
-        <v>84.18811911277291</v>
+        <v>0.08418811911277291</v>
       </c>
       <c r="BH44" t="n">
         <v>761.0329759324582</v>
@@ -8859,13 +8859,13 @@
         <v>0.519642683828383</v>
       </c>
       <c r="BE45" t="n">
-        <v>2080.347916779913</v>
+        <v>2.080347916779913</v>
       </c>
       <c r="BF45" t="n">
-        <v>72704.77607848516</v>
+        <v>72.70477607848517</v>
       </c>
       <c r="BG45" t="n">
-        <v>68.322993604077</v>
+        <v>0.06832299360407701</v>
       </c>
       <c r="BH45" t="n">
         <v>1064.133350183688</v>
@@ -9044,13 +9044,13 @@
         <v>0.739226720261438</v>
       </c>
       <c r="BE46" t="n">
-        <v>1803.572361821152</v>
+        <v>1.803572361821152</v>
       </c>
       <c r="BF46" t="n">
-        <v>49813.58951370534</v>
+        <v>49.81358951370535</v>
       </c>
       <c r="BG46" t="n">
-        <v>90.96646912462749</v>
+        <v>0.0909664691246275</v>
       </c>
       <c r="BH46" t="n">
         <v>547.6038587961334</v>
@@ -9229,13 +9229,13 @@
         <v>0.891906181936322</v>
       </c>
       <c r="BE47" t="n">
-        <v>1563.233988308393</v>
+        <v>1.563233988308393</v>
       </c>
       <c r="BF47" t="n">
-        <v>49415.60931653564</v>
+        <v>49.41560931653564</v>
       </c>
       <c r="BG47" t="n">
-        <v>91.86950982567778</v>
+        <v>0.09186950982567778</v>
       </c>
       <c r="BH47" t="n">
         <v>537.8891147922924</v>
@@ -9414,13 +9414,13 @@
         <v>0.736298419596354</v>
       </c>
       <c r="BE48" t="n">
-        <v>1727.182447385554</v>
+        <v>1.727182447385554</v>
       </c>
       <c r="BF48" t="n">
-        <v>56276.08137299266</v>
+        <v>56.27608137299266</v>
       </c>
       <c r="BG48" t="n">
-        <v>87.61808220891884</v>
+        <v>0.08761808220891884</v>
       </c>
       <c r="BH48" t="n">
         <v>642.2884404021363</v>
@@ -9599,13 +9599,13 @@
         <v>0.659533250666667</v>
       </c>
       <c r="BE49" t="n">
-        <v>2118.768969038877</v>
+        <v>2.118768969038876</v>
       </c>
       <c r="BF49" t="n">
-        <v>78609.92204916544</v>
+        <v>78.60992204916545</v>
       </c>
       <c r="BG49" t="n">
-        <v>114.2772903664339</v>
+        <v>0.1142772903664339</v>
       </c>
       <c r="BH49" t="n">
         <v>687.8875216335649</v>
@@ -9784,13 +9784,13 @@
         <v>0.533526070957096</v>
       </c>
       <c r="BE50" t="n">
-        <v>1305.405133948935</v>
+        <v>1.305405133948935</v>
       </c>
       <c r="BF50" t="n">
-        <v>60858.78779925097</v>
+        <v>60.85878779925097</v>
       </c>
       <c r="BG50" t="n">
-        <v>77.04597268100757</v>
+        <v>0.07704597268100756</v>
       </c>
       <c r="BH50" t="n">
         <v>789.9022581131373</v>
@@ -9969,13 +9969,13 @@
         <v>0.745449478580991</v>
       </c>
       <c r="BE51" t="n">
-        <v>2749.705279828398</v>
+        <v>2.749705279828398</v>
       </c>
       <c r="BF51" t="n">
-        <v>76008.80368696366</v>
+        <v>76.00880368696366</v>
       </c>
       <c r="BG51" t="n">
-        <v>131.1078270933511</v>
+        <v>0.1311078270933511</v>
       </c>
       <c r="BH51" t="n">
         <v>579.7426848729941</v>
@@ -10154,13 +10154,13 @@
         <v>0.844184348484848</v>
       </c>
       <c r="BE52" t="n">
-        <v>2554.237568151246</v>
+        <v>2.554237568151246</v>
       </c>
       <c r="BF52" t="n">
-        <v>80296.6293999513</v>
+        <v>80.29662939995131</v>
       </c>
       <c r="BG52" t="n">
-        <v>152.4967523895981</v>
+        <v>0.1524967523895981</v>
       </c>
       <c r="BH52" t="n">
         <v>526.5464879855921</v>
@@ -10334,10 +10334,10 @@
       </c>
       <c r="BE53" t="inlineStr"/>
       <c r="BF53" t="n">
-        <v>34691.68210591955</v>
+        <v>34.69168210591955</v>
       </c>
       <c r="BG53" t="n">
-        <v>92.71228920458452</v>
+        <v>0.09271228920458452</v>
       </c>
       <c r="BH53" t="n">
         <v>374.1864471641596</v>
@@ -10514,13 +10514,13 @@
         <v>0.994744053177691</v>
       </c>
       <c r="BE54" t="n">
-        <v>2230.482700063978</v>
+        <v>2.230482700063978</v>
       </c>
       <c r="BF54" t="n">
-        <v>38341.14387266885</v>
+        <v>38.34114387266885</v>
       </c>
       <c r="BG54" t="n">
-        <v>91.07493274206992</v>
+        <v>0.09107493274206992</v>
       </c>
       <c r="BH54" t="n">
         <v>420.9845971696014</v>
@@ -10699,13 +10699,13 @@
         <v>0.737201217191601</v>
       </c>
       <c r="BE55" t="n">
-        <v>2700.331914670088</v>
+        <v>2.700331914670088</v>
       </c>
       <c r="BF55" t="n">
-        <v>92268.08188432537</v>
+        <v>92.26808188432537</v>
       </c>
       <c r="BG55" t="n">
-        <v>153.3735609526217</v>
+        <v>0.1533735609526217</v>
       </c>
       <c r="BH55" t="n">
         <v>601.5905304097862</v>
@@ -10884,13 +10884,13 @@
         <v>0.780848745701058</v>
       </c>
       <c r="BE56" t="n">
-        <v>1811.914954031918</v>
+        <v>1.811914954031918</v>
       </c>
       <c r="BF56" t="n">
-        <v>56407.59522824798</v>
+        <v>56.40759522824798</v>
       </c>
       <c r="BG56" t="n">
-        <v>92.6429867997474</v>
+        <v>0.0926429867997474</v>
       </c>
       <c r="BH56" t="n">
         <v>608.8706460876085</v>
@@ -11069,13 +11069,13 @@
         <v>0.608936419471947</v>
       </c>
       <c r="BE57" t="n">
-        <v>1485.071659290358</v>
+        <v>1.485071659290358</v>
       </c>
       <c r="BF57" t="n">
-        <v>62792.70830799232</v>
+        <v>62.79270830799231</v>
       </c>
       <c r="BG57" t="n">
-        <v>86.00555541924115</v>
+        <v>0.08600555541924114</v>
       </c>
       <c r="BH57" t="n">
         <v>730.1006080584458</v>
@@ -11254,13 +11254,13 @@
         <v>0.9247194051332031</v>
       </c>
       <c r="BE58" t="n">
-        <v>1818.05467668072</v>
+        <v>1.81805467668072</v>
       </c>
       <c r="BF58" t="n">
-        <v>55284.08572483942</v>
+        <v>55.28408572483941</v>
       </c>
       <c r="BG58" t="n">
-        <v>106.2801065910518</v>
+        <v>0.1062801065910518</v>
       </c>
       <c r="BH58" t="n">
         <v>520.1734124859641</v>
@@ -11439,13 +11439,13 @@
         <v>0.767365057856673</v>
       </c>
       <c r="BE59" t="n">
-        <v>1468.960643433882</v>
+        <v>1.468960643433882</v>
       </c>
       <c r="BF59" t="n">
-        <v>60805.98725084784</v>
+        <v>60.80598725084783</v>
       </c>
       <c r="BG59" t="n">
-        <v>100.0115293640498</v>
+        <v>0.1000115293640498</v>
       </c>
       <c r="BH59" t="n">
         <v>607.9897751539154</v>
@@ -11624,13 +11624,13 @@
         <v>0.905815394205729</v>
       </c>
       <c r="BE60" t="n">
-        <v>1640.718941643498</v>
+        <v>1.640718941643498</v>
       </c>
       <c r="BF60" t="n">
-        <v>46204.40023861259</v>
+        <v>46.20440023861259</v>
       </c>
       <c r="BG60" t="n">
-        <v>96.820681841672</v>
+        <v>0.09682068184167199</v>
       </c>
       <c r="BH60" t="n">
         <v>477.2162244650299</v>
@@ -11809,13 +11809,13 @@
         <v>1.0241003369709</v>
       </c>
       <c r="BE61" t="n">
-        <v>2324.436326842925</v>
+        <v>2.324436326842925</v>
       </c>
       <c r="BF61" t="n">
-        <v>65896.93642640406</v>
+        <v>65.89693642640407</v>
       </c>
       <c r="BG61" t="n">
-        <v>150.2198334650496</v>
+        <v>0.1502198334650496</v>
       </c>
       <c r="BH61" t="n">
         <v>438.6700138483095</v>
@@ -11994,13 +11994,13 @@
         <v>0.5485383858085811</v>
       </c>
       <c r="BE62" t="n">
-        <v>2271.852849396293</v>
+        <v>2.271852849396293</v>
       </c>
       <c r="BF62" t="n">
-        <v>81219.991100984</v>
+        <v>81.219991100984</v>
       </c>
       <c r="BG62" t="n">
-        <v>90.75866832792745</v>
+        <v>0.09075866832792745</v>
       </c>
       <c r="BH62" t="n">
         <v>894.9006480298004</v>
@@ -12179,13 +12179,13 @@
         <v>0.475137969907407</v>
       </c>
       <c r="BE63" t="n">
-        <v>2097.736888129386</v>
+        <v>2.097736888129386</v>
       </c>
       <c r="BF63" t="n">
-        <v>66593.17142649229</v>
+        <v>66.59317142649229</v>
       </c>
       <c r="BG63" t="n">
-        <v>66.70897453309414</v>
+        <v>0.06670897453309414</v>
       </c>
       <c r="BH63" t="n">
         <v>998.2640550628702</v>
@@ -12364,13 +12364,13 @@
         <v>0.475137969907407</v>
       </c>
       <c r="BE64" t="n">
-        <v>2051.731480905204</v>
+        <v>2.051731480905204</v>
       </c>
       <c r="BF64" t="n">
-        <v>67204.09857723063</v>
+        <v>67.20409857723064</v>
       </c>
       <c r="BG64" t="n">
-        <v>66.70897453309414</v>
+        <v>0.06670897453309414</v>
       </c>
       <c r="BH64" t="n">
         <v>1007.422150431811</v>
@@ -12549,13 +12549,13 @@
         <v>0.993249184926959</v>
       </c>
       <c r="BE65" t="n">
-        <v>1711.270057226029</v>
+        <v>1.71127005722603</v>
       </c>
       <c r="BF65" t="n">
-        <v>64651.41386759904</v>
+        <v>64.65141386759905</v>
       </c>
       <c r="BG65" t="n">
-        <v>140.3287181341011</v>
+        <v>0.1403287181341011</v>
       </c>
       <c r="BH65" t="n">
         <v>460.7140628607237</v>
@@ -12734,13 +12734,13 @@
         <v>1.90429296090126</v>
       </c>
       <c r="BE66" t="n">
-        <v>1264.668813853405</v>
+        <v>1.264668813853405</v>
       </c>
       <c r="BF66" t="n">
-        <v>59173.73389442117</v>
+        <v>59.17373389442116</v>
       </c>
       <c r="BG66" t="n">
-        <v>260.7374490835797</v>
+        <v>0.2607374490835797</v>
       </c>
       <c r="BH66" t="n">
         <v>226.9475831047689</v>
@@ -12919,13 +12919,13 @@
         <v>1.16583652948973</v>
       </c>
       <c r="BE67" t="n">
-        <v>1735.620252135451</v>
+        <v>1.735620252135451</v>
       </c>
       <c r="BF67" t="n">
-        <v>51302.29695978934</v>
+        <v>51.30229695978934</v>
       </c>
       <c r="BG67" t="n">
-        <v>137.0709413665789</v>
+        <v>0.1370709413665789</v>
       </c>
       <c r="BH67" t="n">
         <v>374.2755134553855</v>
@@ -13104,13 +13104,13 @@
         <v>1.36348950458415</v>
       </c>
       <c r="BE68" t="n">
-        <v>1651.892043876882</v>
+        <v>1.651892043876882</v>
       </c>
       <c r="BF68" t="n">
-        <v>46172.17165350541</v>
+        <v>46.1721716535054</v>
       </c>
       <c r="BG68" t="n">
-        <v>142.319283016586</v>
+        <v>0.1423192830165859</v>
       </c>
       <c r="BH68" t="n">
         <v>324.4266741290741</v>
@@ -13289,13 +13289,13 @@
         <v>0.82408405687048</v>
       </c>
       <c r="BE69" t="n">
-        <v>1729.739026459769</v>
+        <v>1.729739026459769</v>
       </c>
       <c r="BF69" t="n">
-        <v>41692.61023831525</v>
+        <v>41.69261023831525</v>
       </c>
       <c r="BG69" t="n">
-        <v>80.06093000193269</v>
+        <v>0.08006093000193269</v>
       </c>
       <c r="BH69" t="n">
         <v>520.7610033671701</v>
@@ -13474,13 +13474,13 @@
         <v>0.535751518300654</v>
       </c>
       <c r="BE70" t="n">
-        <v>1653.302877966243</v>
+        <v>1.653302877966243</v>
       </c>
       <c r="BF70" t="n">
-        <v>54689.10140257988</v>
+        <v>54.68910140257988</v>
       </c>
       <c r="BG70" t="n">
-        <v>68.09229172210588</v>
+        <v>0.06809229172210589</v>
       </c>
       <c r="BH70" t="n">
         <v>803.1614154767136</v>
@@ -13659,13 +13659,13 @@
         <v>0.459120420727745</v>
       </c>
       <c r="BE71" t="n">
-        <v>2245.34879706159</v>
+        <v>2.24534879706159</v>
       </c>
       <c r="BF71" t="n">
-        <v>63852.61085941602</v>
+        <v>63.85261085941602</v>
       </c>
       <c r="BG71" t="n">
-        <v>61.6838561941078</v>
+        <v>0.06168385619410779</v>
       </c>
       <c r="BH71" t="n">
         <v>1035.159193979111</v>
@@ -13844,13 +13844,13 @@
         <v>1.15668780924479</v>
       </c>
       <c r="BE72" t="n">
-        <v>1704.181532420173</v>
+        <v>1.704181532420173</v>
       </c>
       <c r="BF72" t="n">
-        <v>46455.2151410903</v>
+        <v>46.45521514109029</v>
       </c>
       <c r="BG72" t="n">
-        <v>123.2649263881841</v>
+        <v>0.1232649263881841</v>
       </c>
       <c r="BH72" t="n">
         <v>376.872939466935</v>
@@ -14029,13 +14029,13 @@
         <v>1.54303913845144</v>
       </c>
       <c r="BE73" t="n">
-        <v>1771.344004138958</v>
+        <v>1.771344004138958</v>
       </c>
       <c r="BF73" t="n">
-        <v>53177.20031155273</v>
+        <v>53.17720031155272</v>
       </c>
       <c r="BG73" t="n">
-        <v>191.2114171631317</v>
+        <v>0.1912114171631317</v>
       </c>
       <c r="BH73" t="n">
         <v>278.1068259443143</v>
@@ -14214,13 +14214,13 @@
         <v>1.41513398290598</v>
       </c>
       <c r="BE74" t="n">
-        <v>2890.653446677475</v>
+        <v>2.890653446677475</v>
       </c>
       <c r="BF74" t="n">
-        <v>76507.14677495467</v>
+        <v>76.50714677495466</v>
       </c>
       <c r="BG74" t="n">
-        <v>243.3980165400989</v>
+        <v>0.2433980165400989</v>
       </c>
       <c r="BH74" t="n">
         <v>314.3293764776855</v>
@@ -14399,13 +14399,13 @@
         <v>0.708585888888889</v>
       </c>
       <c r="BE75" t="n">
-        <v>2678.379030470969</v>
+        <v>2.678379030470969</v>
       </c>
       <c r="BF75" t="n">
-        <v>80943.94089102797</v>
+        <v>80.94394089102798</v>
       </c>
       <c r="BG75" t="n">
-        <v>120.5138510574179</v>
+        <v>0.1205138510574179</v>
       </c>
       <c r="BH75" t="n">
         <v>671.6567446879022</v>
@@ -14584,13 +14584,13 @@
         <v>0.781730154808959</v>
       </c>
       <c r="BE76" t="n">
-        <v>2020.516390549202</v>
+        <v>2.020516390549202</v>
       </c>
       <c r="BF76" t="n">
-        <v>66138.2937268838</v>
+        <v>66.1382937268838</v>
       </c>
       <c r="BG76" t="n">
-        <v>116.2431558041077</v>
+        <v>0.1162431558041077</v>
       </c>
       <c r="BH76" t="n">
         <v>568.9650566467731</v>
@@ -14769,13 +14769,13 @@
         <v>0.84443941309987</v>
       </c>
       <c r="BE77" t="n">
-        <v>2290.004233178915</v>
+        <v>2.290004233178915</v>
       </c>
       <c r="BF77" t="n">
-        <v>63798.56596163442</v>
+        <v>63.79856596163442</v>
       </c>
       <c r="BG77" t="n">
-        <v>124.8451324330222</v>
+        <v>0.1248451324330223</v>
       </c>
       <c r="BH77" t="n">
         <v>511.0216531338256</v>
@@ -14954,13 +14954,13 @@
         <v>0.8158367908299869</v>
       </c>
       <c r="BE78" t="n">
-        <v>2143.935207599353</v>
+        <v>2.143935207599353</v>
       </c>
       <c r="BF78" t="n">
-        <v>46772.53989798563</v>
+        <v>46.77253989798564</v>
       </c>
       <c r="BG78" t="n">
-        <v>88.70798703209563</v>
+        <v>0.08870798703209562</v>
       </c>
       <c r="BH78" t="n">
         <v>527.2641332855717</v>
@@ -15139,13 +15139,13 @@
         <v>0.830341156785244</v>
       </c>
       <c r="BE79" t="n">
-        <v>3250.436485054538</v>
+        <v>3.250436485054538</v>
       </c>
       <c r="BF79" t="n">
-        <v>59433.53709831833</v>
+        <v>59.43353709831833</v>
       </c>
       <c r="BG79" t="n">
-        <v>113.7751793388308</v>
+        <v>0.1137751793388307</v>
       </c>
       <c r="BH79" t="n">
         <v>522.377002116788</v>
@@ -15324,13 +15324,13 @@
         <v>0.778980451155116</v>
       </c>
       <c r="BE80" t="n">
-        <v>2998.648154876038</v>
+        <v>2.998648154876038</v>
       </c>
       <c r="BF80" t="n">
-        <v>66357.35356277657</v>
+        <v>66.35735356277657</v>
       </c>
       <c r="BG80" t="n">
-        <v>123.3753247448174</v>
+        <v>0.1233753247448174</v>
       </c>
       <c r="BH80" t="n">
         <v>537.8494743582348</v>
@@ -15509,13 +15509,13 @@
         <v>0.860931369189907</v>
       </c>
       <c r="BE81" t="n">
-        <v>2994.186256562353</v>
+        <v>2.994186256562354</v>
       </c>
       <c r="BF81" t="n">
-        <v>71524.31113667959</v>
+        <v>71.5243111366796</v>
       </c>
       <c r="BG81" t="n">
-        <v>142.3646390213997</v>
+        <v>0.1423646390213997</v>
       </c>
       <c r="BH81" t="n">
         <v>502.4022231105318</v>
@@ -15694,13 +15694,13 @@
         <v>0.56359897356091</v>
       </c>
       <c r="BE82" t="n">
-        <v>1986.099449474032</v>
+        <v>1.986099449474032</v>
       </c>
       <c r="BF82" t="n">
-        <v>58036.6638296212</v>
+        <v>58.0366638296212</v>
       </c>
       <c r="BG82" t="n">
-        <v>68.16167495226779</v>
+        <v>0.06816167495226778</v>
       </c>
       <c r="BH82" t="n">
         <v>851.4559519005818</v>
@@ -15879,13 +15879,13 @@
         <v>1.05432551060305</v>
       </c>
       <c r="BE83" t="n">
-        <v>1574.768288150041</v>
+        <v>1.574768288150041</v>
       </c>
       <c r="BF83" t="n">
-        <v>41441.99615258708</v>
+        <v>41.44199615258708</v>
       </c>
       <c r="BG83" t="n">
-        <v>99.14099335271644</v>
+        <v>0.09914099335271642</v>
       </c>
       <c r="BH83" t="n">
         <v>418.0107012358434</v>
@@ -16064,13 +16064,13 @@
         <v>0.939988653135314</v>
       </c>
       <c r="BE84" t="n">
-        <v>1625.698637855855</v>
+        <v>1.625698637855855</v>
       </c>
       <c r="BF84" t="n">
-        <v>49102.86937521602</v>
+        <v>49.10286937521602</v>
       </c>
       <c r="BG84" t="n">
-        <v>97.56221518246466</v>
+        <v>0.09756221518246466</v>
       </c>
       <c r="BH84" t="n">
         <v>503.298016382489</v>
@@ -16249,13 +16249,13 @@
         <v>0.638802563523248</v>
       </c>
       <c r="BE85" t="n">
-        <v>2261.410104794486</v>
+        <v>2.261410104794487</v>
       </c>
       <c r="BF85" t="n">
-        <v>63281.75428570905</v>
+        <v>63.28175428570905</v>
       </c>
       <c r="BG85" t="n">
-        <v>84.14982775568258</v>
+        <v>0.08414982775568258</v>
       </c>
       <c r="BH85" t="n">
         <v>752.0128795680829</v>
@@ -16434,13 +16434,13 @@
         <v>0.744430595751634</v>
       </c>
       <c r="BE86" t="n">
-        <v>2131.678007547578</v>
+        <v>2.131678007547578</v>
       </c>
       <c r="BF86" t="n">
-        <v>65226.38295327906</v>
+        <v>65.22638295327906</v>
       </c>
       <c r="BG86" t="n">
-        <v>100.5776032211469</v>
+        <v>0.1005776032211469</v>
       </c>
       <c r="BH86" t="n">
         <v>648.5179688549674</v>
@@ -16619,13 +16619,13 @@
         <v>1.02055795016502</v>
       </c>
       <c r="BE87" t="n">
-        <v>2723.142473493238</v>
+        <v>2.723142473493239</v>
       </c>
       <c r="BF87" t="n">
-        <v>73543.63492686352</v>
+        <v>73.54363492686352</v>
       </c>
       <c r="BG87" t="n">
-        <v>169.4962030644245</v>
+        <v>0.1694962030644245</v>
       </c>
       <c r="BH87" t="n">
         <v>433.8954713865184</v>
@@ -16804,13 +16804,13 @@
         <v>1.32171089713542</v>
       </c>
       <c r="BE88" t="n">
-        <v>2165.437559626952</v>
+        <v>2.165437559626953</v>
       </c>
       <c r="BF88" t="n">
-        <v>43524.89670002637</v>
+        <v>43.52489670002637</v>
       </c>
       <c r="BG88" t="n">
-        <v>130.0815175398405</v>
+        <v>0.1300815175398405</v>
       </c>
       <c r="BH88" t="n">
         <v>334.5970859134222</v>
@@ -16995,13 +16995,13 @@
         <v>0.3022689226426593</v>
       </c>
       <c r="BE89" t="n">
-        <v>2273.110803333757</v>
+        <v>2.273110803333757</v>
       </c>
       <c r="BF89" t="n">
-        <v>134993.6057389324</v>
+        <v>134.9936057389324</v>
       </c>
       <c r="BG89" t="n">
-        <v>88.48636680398482</v>
+        <v>0.08848636680398482</v>
       </c>
       <c r="BH89" t="n">
         <v>1525.586489927545</v>
@@ -17186,13 +17186,13 @@
         <v>1.663948688200762</v>
       </c>
       <c r="BE90" t="n">
-        <v>2562.349769016561</v>
+        <v>2.562349769016561</v>
       </c>
       <c r="BF90" t="n">
-        <v>141122.6797838226</v>
+        <v>141.1226797838225</v>
       </c>
       <c r="BG90" t="n">
-        <v>501.4469628804882</v>
+        <v>0.5014469628804882</v>
       </c>
       <c r="BH90" t="n">
         <v>281.4309193801157</v>
@@ -17377,13 +17377,13 @@
         <v>0.3625060659950419</v>
       </c>
       <c r="BE91" t="n">
-        <v>2747.689268163115</v>
+        <v>2.747689268163116</v>
       </c>
       <c r="BF91" t="n">
-        <v>124133.9472150039</v>
+        <v>124.1339472150039</v>
       </c>
       <c r="BG91" t="n">
-        <v>95.55605740821525</v>
+        <v>0.09555605740821525</v>
       </c>
       <c r="BH91" t="n">
         <v>1299.069369142178</v>
@@ -17568,13 +17568,13 @@
         <v>0.4849510454859731</v>
       </c>
       <c r="BE92" t="n">
-        <v>2638.257036105743</v>
+        <v>2.638257036105744</v>
       </c>
       <c r="BF92" t="n">
-        <v>114464.4073918296</v>
+        <v>114.4644073918296</v>
       </c>
       <c r="BG92" t="n">
-        <v>119.5499967120293</v>
+        <v>0.1195499967120293</v>
       </c>
       <c r="BH92" t="n">
         <v>957.4605649513329</v>
@@ -17759,13 +17759,13 @@
         <v>0.3547881208221685</v>
       </c>
       <c r="BE93" t="n">
-        <v>2205.905999210828</v>
+        <v>2.205905999210827</v>
       </c>
       <c r="BF93" t="n">
-        <v>134610.8772447198</v>
+        <v>134.6108772447198</v>
       </c>
       <c r="BG93" t="n">
-        <v>100.621858720207</v>
+        <v>0.100621858720207</v>
       </c>
       <c r="BH93" t="n">
         <v>1337.789611092595</v>
@@ -17950,13 +17950,13 @@
         <v>0.3949439937897002</v>
       </c>
       <c r="BE94" t="n">
-        <v>2899.244513121407</v>
+        <v>2.899244513121407</v>
       </c>
       <c r="BF94" t="n">
-        <v>145509.8595795598</v>
+        <v>145.5098595795598</v>
       </c>
       <c r="BG94" t="n">
-        <v>119.1322287326202</v>
+        <v>0.1191322287326202</v>
       </c>
       <c r="BH94" t="n">
         <v>1221.414734934082</v>
@@ -18141,13 +18141,13 @@
         <v>0.7511820368610592</v>
       </c>
       <c r="BE95" t="n">
-        <v>3639.814907180162</v>
+        <v>3.639814907180162</v>
       </c>
       <c r="BF95" t="n">
-        <v>162100.5166131244</v>
+        <v>162.1005166131244</v>
       </c>
       <c r="BG95" t="n">
-        <v>246.2501351629302</v>
+        <v>0.2462501351629302</v>
       </c>
       <c r="BH95" t="n">
         <v>658.2758482787081</v>
@@ -18332,13 +18332,13 @@
         <v>1.381135177865805</v>
       </c>
       <c r="BE96" t="n">
-        <v>2754.165199655664</v>
+        <v>2.754165199655664</v>
       </c>
       <c r="BF96" t="n">
-        <v>115432.612977339</v>
+        <v>115.432612977339</v>
       </c>
       <c r="BG96" t="n">
-        <v>344.6635811046561</v>
+        <v>0.3446635811046561</v>
       </c>
       <c r="BH96" t="n">
         <v>334.9138676252779</v>
@@ -18523,13 +18523,13 @@
         <v>2.442251007971658</v>
       </c>
       <c r="BE97" t="n">
-        <v>2635.851161810385</v>
+        <v>2.635851161810385</v>
       </c>
       <c r="BF97" t="n">
-        <v>186370.8247181081</v>
+        <v>186.3708247181081</v>
       </c>
       <c r="BG97" t="n">
-        <v>971.3779599734123</v>
+        <v>0.9713779599734124</v>
       </c>
       <c r="BH97" t="n">
         <v>191.862315594652</v>
@@ -18714,13 +18714,13 @@
         <v>2.513685244069834</v>
       </c>
       <c r="BE98" t="n">
-        <v>2379.812101557392</v>
+        <v>2.379812101557392</v>
       </c>
       <c r="BF98" t="n">
-        <v>133643.1271950471</v>
+        <v>133.6431271950471</v>
       </c>
       <c r="BG98" t="n">
-        <v>736.9732006727197</v>
+        <v>0.7369732006727198</v>
       </c>
       <c r="BH98" t="n">
         <v>181.3405522386102</v>
@@ -18905,13 +18905,13 @@
         <v>0.435002842237245</v>
       </c>
       <c r="BE99" t="n">
-        <v>1937.192235493844</v>
+        <v>1.937192235493844</v>
       </c>
       <c r="BF99" t="n">
-        <v>108080.729022015</v>
+        <v>108.080729022015</v>
       </c>
       <c r="BG99" t="n">
-        <v>100.2304190887461</v>
+        <v>0.1002304190887461</v>
       </c>
       <c r="BH99" t="n">
         <v>1078.322629044563</v>
@@ -19096,13 +19096,13 @@
         <v>1.128182611778521</v>
       </c>
       <c r="BE100" t="n">
-        <v>1937.567807703534</v>
+        <v>1.937567807703533</v>
       </c>
       <c r="BF100" t="n">
-        <v>127753.0493515518</v>
+        <v>127.7530493515518</v>
       </c>
       <c r="BG100" t="n">
-        <v>314.468218366653</v>
+        <v>0.314468218366653</v>
       </c>
       <c r="BH100" t="n">
         <v>406.251067325979</v>
@@ -19287,13 +19287,13 @@
         <v>0.7365982038830503</v>
       </c>
       <c r="BE101" t="n">
-        <v>4431.249649472029</v>
+        <v>4.431249649472029</v>
       </c>
       <c r="BF101" t="n">
-        <v>157281.7308080371</v>
+        <v>157.2817308080371</v>
       </c>
       <c r="BG101" t="n">
-        <v>230.407831176971</v>
+        <v>0.230407831176971</v>
       </c>
       <c r="BH101" t="n">
         <v>682.6231990666696</v>
@@ -19478,13 +19478,13 @@
         <v>0.6125897805332587</v>
       </c>
       <c r="BE102" t="n">
-        <v>2369.266782339464</v>
+        <v>2.369266782339464</v>
       </c>
       <c r="BF102" t="n">
-        <v>148213.9105150992</v>
+        <v>148.2139105150992</v>
       </c>
       <c r="BG102" t="n">
-        <v>189.9408842031573</v>
+        <v>0.1899408842031573</v>
       </c>
       <c r="BH102" t="n">
         <v>780.3159974583056</v>
@@ -19669,13 +19669,13 @@
         <v>0.4058516935832551</v>
       </c>
       <c r="BE103" t="n">
-        <v>2767.201366776576</v>
+        <v>2.767201366776576</v>
       </c>
       <c r="BF103" t="n">
-        <v>133337.1549183661</v>
+        <v>133.3371549183661</v>
       </c>
       <c r="BG103" t="n">
-        <v>115.1976622107068</v>
+        <v>0.1151976622107068</v>
       </c>
       <c r="BH103" t="n">
         <v>1157.464069665586</v>
@@ -19860,13 +19860,13 @@
         <v>0.8893053640303116</v>
       </c>
       <c r="BE104" t="n">
-        <v>2793.068603846922</v>
+        <v>2.793068603846922</v>
       </c>
       <c r="BF104" t="n">
-        <v>135464.8469089234</v>
+        <v>135.4648469089233</v>
       </c>
       <c r="BG104" t="n">
-        <v>261.3183231977535</v>
+        <v>0.2613183231977535</v>
       </c>
       <c r="BH104" t="n">
         <v>518.3901582225059</v>
@@ -20051,13 +20051,13 @@
         <v>1.433819373048095</v>
       </c>
       <c r="BE105" t="n">
-        <v>2872.854831093412</v>
+        <v>2.872854831093412</v>
       </c>
       <c r="BF105" t="n">
-        <v>140264.4284387566</v>
+        <v>140.2644284387566</v>
       </c>
       <c r="BG105" t="n">
-        <v>416.5641702066033</v>
+        <v>0.4165641702066033</v>
       </c>
       <c r="BH105" t="n">
         <v>336.7174578869558</v>
@@ -20242,13 +20242,13 @@
         <v>0.4225314752105393</v>
       </c>
       <c r="BE106" t="n">
-        <v>2999.907207031169</v>
+        <v>2.999907207031169</v>
       </c>
       <c r="BF106" t="n">
-        <v>126253.1036318729</v>
+        <v>126.2531036318729</v>
       </c>
       <c r="BG106" t="n">
-        <v>113.7859568730906</v>
+        <v>0.1137859568730906</v>
       </c>
       <c r="BH106" t="n">
         <v>1109.566655687461</v>
@@ -20433,13 +20433,13 @@
         <v>0.4239581226118181</v>
       </c>
       <c r="BE107" t="n">
-        <v>2588.902949996616</v>
+        <v>2.588902949996617</v>
       </c>
       <c r="BF107" t="n">
-        <v>134481.2445048961</v>
+        <v>134.4812445048961</v>
       </c>
       <c r="BG107" t="n">
-        <v>121.3665020885663</v>
+        <v>0.1213665020885663</v>
       </c>
       <c r="BH107" t="n">
         <v>1108.058996433459</v>
@@ -20624,13 +20624,13 @@
         <v>2.296553217814438</v>
       </c>
       <c r="BE108" t="n">
-        <v>2195.244308829524</v>
+        <v>2.195244308829523</v>
       </c>
       <c r="BF108" t="n">
-        <v>122108.1274983239</v>
+        <v>122.1081274983239</v>
       </c>
       <c r="BG108" t="n">
-        <v>602.4469470906693</v>
+        <v>0.6024469470906693</v>
       </c>
       <c r="BH108" t="n">
         <v>202.6869388051633</v>
@@ -20815,13 +20815,13 @@
         <v>2.206920483298215</v>
       </c>
       <c r="BE109" t="n">
-        <v>2371.581729527561</v>
+        <v>2.371581729527561</v>
       </c>
       <c r="BF109" t="n">
-        <v>139808.4821573612</v>
+        <v>139.8084821573613</v>
       </c>
       <c r="BG109" t="n">
-        <v>648.5978477080954</v>
+        <v>0.6485978477080955</v>
       </c>
       <c r="BH109" t="n">
         <v>215.5549585176587</v>
@@ -21006,13 +21006,13 @@
         <v>2.0718698133459</v>
       </c>
       <c r="BE110" t="n">
-        <v>2120.569899826035</v>
+        <v>2.120569899826035</v>
       </c>
       <c r="BF110" t="n">
-        <v>130817.7853020215</v>
+        <v>130.8177853020215</v>
       </c>
       <c r="BG110" t="n">
-        <v>575.069649383158</v>
+        <v>0.575069649383158</v>
       </c>
       <c r="BH110" t="n">
         <v>227.4816371240279</v>
@@ -21197,13 +21197,13 @@
         <v>1.718324936833187</v>
       </c>
       <c r="BE111" t="n">
-        <v>3066.512007482434</v>
+        <v>3.066512007482434</v>
       </c>
       <c r="BF111" t="n">
-        <v>130374.7394486637</v>
+        <v>130.3747394486637</v>
       </c>
       <c r="BG111" t="n">
-        <v>489.434786636057</v>
+        <v>0.4894347866360571</v>
       </c>
       <c r="BH111" t="n">
         <v>266.3781631557998</v>
@@ -21388,13 +21388,13 @@
         <v>0.7330294163502471</v>
       </c>
       <c r="BE112" t="n">
-        <v>3515.637037094179</v>
+        <v>3.515637037094179</v>
       </c>
       <c r="BF112" t="n">
-        <v>153421.6160214485</v>
+        <v>153.4216160214486</v>
       </c>
       <c r="BG112" t="n">
-        <v>227.5609519700245</v>
+        <v>0.2275609519700245</v>
       </c>
       <c r="BH112" t="n">
         <v>674.2000975705974</v>
@@ -21579,13 +21579,13 @@
         <v>0.3719852691735669</v>
       </c>
       <c r="BE113" t="n">
-        <v>2469.291967965981</v>
+        <v>2.469291967965981</v>
       </c>
       <c r="BF113" t="n">
-        <v>119195.3738709075</v>
+        <v>119.1953738709075</v>
       </c>
       <c r="BG113" t="n">
-        <v>95.91448322866695</v>
+        <v>0.09591448322866696</v>
       </c>
       <c r="BH113" t="n">
         <v>1242.725497323873</v>
@@ -21770,13 +21770,13 @@
         <v>1.116051620086352</v>
       </c>
       <c r="BE114" t="n">
-        <v>2429.99367207335</v>
+        <v>2.42999367207335</v>
       </c>
       <c r="BF114" t="n">
-        <v>135315.0056788815</v>
+        <v>135.3150056788816</v>
       </c>
       <c r="BG114" t="n">
-        <v>314.4638401563245</v>
+        <v>0.3144638401563246</v>
       </c>
       <c r="BH114" t="n">
         <v>430.3038645448536</v>
@@ -21961,13 +21961,13 @@
         <v>1.032273647779503</v>
       </c>
       <c r="BE115" t="n">
-        <v>3012.101624121943</v>
+        <v>3.012101624121943</v>
       </c>
       <c r="BF115" t="n">
-        <v>140221.9433572833</v>
+        <v>140.2219433572834</v>
       </c>
       <c r="BG115" t="n">
-        <v>297.0048736509277</v>
+        <v>0.2970048736509278</v>
       </c>
       <c r="BH115" t="n">
         <v>472.1200081116762</v>
@@ -22152,13 +22152,13 @@
         <v>0.9959949821321988</v>
       </c>
       <c r="BE116" t="n">
-        <v>4886.608187366623</v>
+        <v>4.886608187366623</v>
       </c>
       <c r="BF116" t="n">
-        <v>140650.5272762413</v>
+        <v>140.6505272762413</v>
       </c>
       <c r="BG116" t="n">
-        <v>291.1866620672897</v>
+        <v>0.2911866620672897</v>
       </c>
       <c r="BH116" t="n">
         <v>483.0253085003554</v>
@@ -22343,13 +22343,13 @@
         <v>1.294556897594681</v>
       </c>
       <c r="BE117" t="n">
-        <v>2753.295278959289</v>
+        <v>2.753295278959289</v>
       </c>
       <c r="BF117" t="n">
-        <v>110850.3111923048</v>
+        <v>110.8503111923048</v>
       </c>
       <c r="BG117" t="n">
-        <v>298.1906883143227</v>
+        <v>0.2981906883143227</v>
       </c>
       <c r="BH117" t="n">
         <v>371.7430340261248</v>
@@ -22534,13 +22534,13 @@
         <v>1.294556897594681</v>
       </c>
       <c r="BE118" t="n">
-        <v>2753.295278959289</v>
+        <v>2.753295278959289</v>
       </c>
       <c r="BF118" t="n">
-        <v>110850.3111923048</v>
+        <v>110.8503111923048</v>
       </c>
       <c r="BG118" t="n">
-        <v>298.1906883143227</v>
+        <v>0.2981906883143227</v>
       </c>
       <c r="BH118" t="n">
         <v>371.7430340261248</v>
@@ -22725,13 +22725,13 @@
         <v>0.7330305807834134</v>
       </c>
       <c r="BE119" t="n">
-        <v>3326.850351224271</v>
+        <v>3.32685035122427</v>
       </c>
       <c r="BF119" t="n">
-        <v>128510.5915976078</v>
+        <v>128.5105915976078</v>
       </c>
       <c r="BG119" t="n">
-        <v>190.9488702678472</v>
+        <v>0.1909488702678472</v>
       </c>
       <c r="BH119" t="n">
         <v>673.0104839968092</v>
@@ -22916,13 +22916,13 @@
         <v>1.190130963299714</v>
       </c>
       <c r="BE120" t="n">
-        <v>3652.366005865274</v>
+        <v>3.652366005865273</v>
       </c>
       <c r="BF120" t="n">
-        <v>173868.8221141171</v>
+        <v>173.8688221141171</v>
       </c>
       <c r="BG120" t="n">
-        <v>424.936021290441</v>
+        <v>0.424936021290441</v>
       </c>
       <c r="BH120" t="n">
         <v>409.1647057505604</v>
@@ -23107,13 +23107,13 @@
         <v>1.190130963299714</v>
       </c>
       <c r="BE121" t="n">
-        <v>3652.366005865274</v>
+        <v>3.652366005865273</v>
       </c>
       <c r="BF121" t="n">
-        <v>173868.8221141171</v>
+        <v>173.8688221141171</v>
       </c>
       <c r="BG121" t="n">
-        <v>424.936021290441</v>
+        <v>0.424936021290441</v>
       </c>
       <c r="BH121" t="n">
         <v>409.1647057505604</v>
@@ -23298,13 +23298,13 @@
         <v>0.70388853315343</v>
       </c>
       <c r="BE122" t="n">
-        <v>3309.760277186539</v>
+        <v>3.309760277186538</v>
       </c>
       <c r="BF122" t="n">
-        <v>126088.9866039253</v>
+        <v>126.0889866039252</v>
       </c>
       <c r="BG122" t="n">
-        <v>186.5608181721887</v>
+        <v>0.1865608181721887</v>
       </c>
       <c r="BH122" t="n">
         <v>675.8599573011616</v>
@@ -23489,13 +23489,13 @@
         <v>1.706487181309719</v>
       </c>
       <c r="BE123" t="n">
-        <v>3855.984342568878</v>
+        <v>3.855984342568878</v>
       </c>
       <c r="BF123" t="n">
-        <v>138235.7685802533</v>
+        <v>138.2357685802533</v>
       </c>
       <c r="BG123" t="n">
-        <v>488.5371436014495</v>
+        <v>0.4885371436014496</v>
       </c>
       <c r="BH123" t="n">
         <v>282.958563930661</v>
@@ -23680,13 +23680,13 @@
         <v>1.24432515516913</v>
       </c>
       <c r="BE124" t="n">
-        <v>3332.925651824539</v>
+        <v>3.332925651824539</v>
       </c>
       <c r="BF124" t="n">
-        <v>156266.9383954623</v>
+        <v>156.2669383954623</v>
       </c>
       <c r="BG124" t="n">
-        <v>399.0682368682052</v>
+        <v>0.3990682368682052</v>
       </c>
       <c r="BH124" t="n">
         <v>391.5794943286114</v>
@@ -23871,13 +23871,13 @@
         <v>1.528358225791803</v>
       </c>
       <c r="BE125" t="n">
-        <v>2307.284769426641</v>
+        <v>2.307284769426641</v>
       </c>
       <c r="BF125" t="n">
-        <v>118151.6372200387</v>
+        <v>118.1516372200387</v>
       </c>
       <c r="BG125" t="n">
-        <v>372.1584096024218</v>
+        <v>0.3721584096024217</v>
       </c>
       <c r="BH125" t="n">
         <v>317.4767361733422</v>
@@ -24062,13 +24062,13 @@
         <v>0.6059605665087811</v>
       </c>
       <c r="BE126" t="n">
-        <v>2966.946505276404</v>
+        <v>2.966946505276404</v>
       </c>
       <c r="BF126" t="n">
-        <v>132789.3671794441</v>
+        <v>132.7893671794441</v>
       </c>
       <c r="BG126" t="n">
-        <v>162.3552796451581</v>
+        <v>0.1623552796451581</v>
       </c>
       <c r="BH126" t="n">
         <v>817.8937418583928</v>
@@ -24253,13 +24253,13 @@
         <v>0.67413284412384</v>
       </c>
       <c r="BE127" t="n">
-        <v>3487.073324331464</v>
+        <v>3.487073324331464</v>
       </c>
       <c r="BF127" t="n">
-        <v>134202.5316348755</v>
+        <v>134.2025316348755</v>
       </c>
       <c r="BG127" t="n">
-        <v>186.3290222711894</v>
+        <v>0.1863290222711894</v>
       </c>
       <c r="BH127" t="n">
         <v>720.2449194390807</v>
@@ -24444,13 +24444,13 @@
         <v>1.445586054889317</v>
       </c>
       <c r="BE128" t="n">
-        <v>3859.533583523428</v>
+        <v>3.859533583523428</v>
       </c>
       <c r="BF128" t="n">
-        <v>146773.4804419995</v>
+        <v>146.7734804419995</v>
       </c>
       <c r="BG128" t="n">
-        <v>439.2005902239814</v>
+        <v>0.4392005902239814</v>
       </c>
       <c r="BH128" t="n">
         <v>334.1832495424213</v>
@@ -24635,13 +24635,13 @@
         <v>1.818650572788979</v>
       </c>
       <c r="BE129" t="n">
-        <v>3675.873944413487</v>
+        <v>3.675873944413487</v>
       </c>
       <c r="BF129" t="n">
-        <v>156929.0001240953</v>
+        <v>156.9290001240953</v>
       </c>
       <c r="BG129" t="n">
-        <v>584.7214351624981</v>
+        <v>0.5847214351624981</v>
       </c>
       <c r="BH129" t="n">
         <v>268.3824992331325</v>
@@ -24826,13 +24826,13 @@
         <v>1.236769225312605</v>
       </c>
       <c r="BE130" t="n">
-        <v>3771.495585441185</v>
+        <v>3.771495585441185</v>
       </c>
       <c r="BF130" t="n">
-        <v>161889.635632338</v>
+        <v>161.889635632338</v>
       </c>
       <c r="BG130" t="n">
-        <v>406.8493951011535</v>
+        <v>0.4068493951011535</v>
       </c>
       <c r="BH130" t="n">
         <v>397.9104739533605</v>
@@ -25017,13 +25017,13 @@
         <v>1.264200753020895</v>
       </c>
       <c r="BE131" t="n">
-        <v>2767.649227576971</v>
+        <v>2.767649227576972</v>
       </c>
       <c r="BF131" t="n">
-        <v>111162.0750906621</v>
+        <v>111.1620750906621</v>
       </c>
       <c r="BG131" t="n">
-        <v>337.2710106638011</v>
+        <v>0.3372710106638011</v>
       </c>
       <c r="BH131" t="n">
         <v>329.5927357405492</v>
@@ -25208,13 +25208,13 @@
         <v>0.6203181408041061</v>
       </c>
       <c r="BE132" t="n">
-        <v>2667.01832885668</v>
+        <v>2.667018328856681</v>
       </c>
       <c r="BF132" t="n">
-        <v>144407.1534170367</v>
+        <v>144.4071534170367</v>
       </c>
       <c r="BG132" t="n">
-        <v>193.2594943946435</v>
+        <v>0.1932594943946435</v>
       </c>
       <c r="BH132" t="n">
         <v>747.2189341557086</v>
@@ -25399,13 +25399,13 @@
         <v>0.6203181408041061</v>
       </c>
       <c r="BE133" t="n">
-        <v>2667.01832885668</v>
+        <v>2.667018328856681</v>
       </c>
       <c r="BF133" t="n">
-        <v>144407.1534170367</v>
+        <v>144.4071534170367</v>
       </c>
       <c r="BG133" t="n">
-        <v>193.2594943946435</v>
+        <v>0.1932594943946435</v>
       </c>
       <c r="BH133" t="n">
         <v>747.2189341557086</v>
@@ -25590,13 +25590,13 @@
         <v>1.549984801394928</v>
       </c>
       <c r="BE134" t="n">
-        <v>3626.928985621702</v>
+        <v>3.626928985621702</v>
       </c>
       <c r="BF134" t="n">
-        <v>125601.6617616408</v>
+        <v>125.6016617616408</v>
       </c>
       <c r="BG134" t="n">
-        <v>395.8015635726782</v>
+        <v>0.3958015635726783</v>
       </c>
       <c r="BH134" t="n">
         <v>317.3349307362639</v>
@@ -25781,13 +25781,13 @@
         <v>0.8285671225617766</v>
       </c>
       <c r="BE135" t="n">
-        <v>3422.023655820771</v>
+        <v>3.42202365582077</v>
       </c>
       <c r="BF135" t="n">
-        <v>153648.7572900207</v>
+        <v>153.6487572900207</v>
       </c>
       <c r="BG135" t="n">
-        <v>257.9721767789777</v>
+        <v>0.2579721767789777</v>
       </c>
       <c r="BH135" t="n">
         <v>595.6020498352506</v>
@@ -25972,13 +25972,13 @@
         <v>3.752305574824123</v>
       </c>
       <c r="BE136" t="n">
-        <v>2957.9939499805</v>
+        <v>2.9579939499805</v>
       </c>
       <c r="BF136" t="n">
-        <v>129957.0950195319</v>
+        <v>129.9570950195319</v>
       </c>
       <c r="BG136" t="n">
-        <v>984.908331811914</v>
+        <v>0.984908331811914</v>
       </c>
       <c r="BH136" t="n">
         <v>131.9484167429599</v>
@@ -26163,13 +26163,13 @@
         <v>2.003502733491316</v>
       </c>
       <c r="BE137" t="n">
-        <v>1947.483713072644</v>
+        <v>1.947483713072644</v>
       </c>
       <c r="BF137" t="n">
-        <v>122184.6360713435</v>
+        <v>122.1846360713435</v>
       </c>
       <c r="BG137" t="n">
-        <v>531.2872384618877</v>
+        <v>0.5312872384618876</v>
       </c>
       <c r="BH137" t="n">
         <v>229.9784885198377</v>
@@ -26354,13 +26354,13 @@
         <v>0.4976190619757426</v>
       </c>
       <c r="BE138" t="n">
-        <v>2038.052013688129</v>
+        <v>2.038052013688129</v>
       </c>
       <c r="BF138" t="n">
-        <v>115814.211862462</v>
+        <v>115.814211862462</v>
       </c>
       <c r="BG138" t="n">
-        <v>125.2576192118186</v>
+        <v>0.1252576192118186</v>
       </c>
       <c r="BH138" t="n">
         <v>924.6081203779931</v>
@@ -26545,13 +26545,13 @@
         <v>0.442454971215987</v>
       </c>
       <c r="BE139" t="n">
-        <v>2816.066621298269</v>
+        <v>2.816066621298269</v>
       </c>
       <c r="BF139" t="n">
-        <v>146355.3882512526</v>
+        <v>146.3553882512526</v>
       </c>
       <c r="BG139" t="n">
-        <v>132.8280183195209</v>
+        <v>0.1328280183195209</v>
       </c>
       <c r="BH139" t="n">
         <v>1101.841238790383</v>
@@ -26736,13 +26736,13 @@
         <v>1.170421599484877</v>
       </c>
       <c r="BE140" t="n">
-        <v>4155.314276894092</v>
+        <v>4.155314276894092</v>
       </c>
       <c r="BF140" t="n">
-        <v>144242.5670969987</v>
+        <v>144.2425670969987</v>
       </c>
       <c r="BG140" t="n">
-        <v>336.8499551025584</v>
+        <v>0.3368499551025584</v>
       </c>
       <c r="BH140" t="n">
         <v>428.210141969834</v>
@@ -26927,13 +26927,13 @@
         <v>1.034293220205778</v>
       </c>
       <c r="BE141" t="n">
-        <v>9247.567853121815</v>
+        <v>9.247567853121815</v>
       </c>
       <c r="BF141" t="n">
-        <v>155634.5654536335</v>
+        <v>155.6345654536335</v>
       </c>
       <c r="BG141" t="n">
-        <v>323.3923108510388</v>
+        <v>0.3233923108510388</v>
       </c>
       <c r="BH141" t="n">
         <v>481.2562334709375</v>
@@ -27118,13 +27118,13 @@
         <v>0.9413367540650814</v>
       </c>
       <c r="BE142" t="n">
-        <v>2494.199987467023</v>
+        <v>2.494199987467023</v>
       </c>
       <c r="BF142" t="n">
-        <v>121883.136199759</v>
+        <v>121.883136199759</v>
       </c>
       <c r="BG142" t="n">
-        <v>244.5600833511928</v>
+        <v>0.2445600833511928</v>
       </c>
       <c r="BH142" t="n">
         <v>498.3770635403839</v>
@@ -27309,13 +27309,13 @@
         <v>0.4332464644027982</v>
       </c>
       <c r="BE143" t="n">
-        <v>2769.312656787985</v>
+        <v>2.769312656787986</v>
       </c>
       <c r="BF143" t="n">
-        <v>134283.6821757779</v>
+        <v>134.2836821757778</v>
       </c>
       <c r="BG143" t="n">
-        <v>122.1407759333642</v>
+        <v>0.1221407759333641</v>
       </c>
       <c r="BH143" t="n">
         <v>1099.417300648544</v>
@@ -27500,13 +27500,13 @@
         <v>0.3301460673610775</v>
       </c>
       <c r="BE144" t="n">
-        <v>2808.967940938339</v>
+        <v>2.808967940938339</v>
       </c>
       <c r="BF144" t="n">
-        <v>147344.793628725</v>
+        <v>147.344793628725</v>
       </c>
       <c r="BG144" t="n">
-        <v>102.4514079588275</v>
+        <v>0.1024514079588275</v>
       </c>
       <c r="BH144" t="n">
         <v>1438.191983539542</v>
@@ -27691,13 +27691,13 @@
         <v>0.4090062180236554</v>
       </c>
       <c r="BE145" t="n">
-        <v>2748.330291734374</v>
+        <v>2.748330291734374</v>
       </c>
       <c r="BF145" t="n">
-        <v>137751.0746218444</v>
+        <v>137.7510746218445</v>
       </c>
       <c r="BG145" t="n">
-        <v>120.3087575004124</v>
+        <v>0.1203087575004124</v>
       </c>
       <c r="BH145" t="n">
         <v>1144.979613153866</v>
@@ -27882,13 +27882,13 @@
         <v>0.5453809105310884</v>
       </c>
       <c r="BE146" t="n">
-        <v>2749.420947265438</v>
+        <v>2.749420947265438</v>
       </c>
       <c r="BF146" t="n">
-        <v>142004.9960833589</v>
+        <v>142.0049960833589</v>
       </c>
       <c r="BG146" t="n">
-        <v>163.2658646144916</v>
+        <v>0.1632658646144916</v>
       </c>
       <c r="BH146" t="n">
         <v>869.777625706791</v>
@@ -28073,13 +28073,13 @@
         <v>0.421627376985528</v>
       </c>
       <c r="BE147" t="n">
-        <v>2978.536938054128</v>
+        <v>2.978536938054128</v>
       </c>
       <c r="BF147" t="n">
-        <v>121660.5225264648</v>
+        <v>121.6605225264648</v>
       </c>
       <c r="BG147" t="n">
-        <v>111.7265736201473</v>
+        <v>0.1117265736201473</v>
       </c>
       <c r="BH147" t="n">
         <v>1088.913036392679</v>
@@ -28264,13 +28264,13 @@
         <v>0.6299664353692545</v>
       </c>
       <c r="BE148" t="n">
-        <v>3389.107084357813</v>
+        <v>3.389107084357813</v>
       </c>
       <c r="BF148" t="n">
-        <v>126819.0950058426</v>
+        <v>126.8190950058426</v>
       </c>
       <c r="BG148" t="n">
-        <v>170.2599768628932</v>
+        <v>0.1702599768628932</v>
       </c>
       <c r="BH148" t="n">
         <v>744.855586982532</v>
@@ -28455,13 +28455,13 @@
         <v>0.3602235709573822</v>
       </c>
       <c r="BE149" t="n">
-        <v>2277.283663149553</v>
+        <v>2.277283663149553</v>
       </c>
       <c r="BF149" t="n">
-        <v>102445.7483107241</v>
+        <v>102.4457483107241</v>
       </c>
       <c r="BG149" t="n">
-        <v>78.90365227446225</v>
+        <v>0.07890365227446225</v>
       </c>
       <c r="BH149" t="n">
         <v>1298.365099176549</v>
@@ -28646,13 +28646,13 @@
         <v>0.3894930957229775</v>
       </c>
       <c r="BE150" t="n">
-        <v>2391.202896295107</v>
+        <v>2.391202896295107</v>
       </c>
       <c r="BF150" t="n">
-        <v>149040.7090683407</v>
+        <v>149.0407090683408</v>
       </c>
       <c r="BG150" t="n">
-        <v>123.1773494420704</v>
+        <v>0.1231773494420704</v>
       </c>
       <c r="BH150" t="n">
         <v>1209.968470205098</v>
@@ -28837,13 +28837,13 @@
         <v>0.4436594649764164</v>
       </c>
       <c r="BE151" t="n">
-        <v>1934.834464052721</v>
+        <v>1.934834464052721</v>
       </c>
       <c r="BF151" t="n">
-        <v>121974.0238789016</v>
+        <v>121.9740238789016</v>
       </c>
       <c r="BG151" t="n">
-        <v>116.5180938818814</v>
+        <v>0.1165180938818813</v>
       </c>
       <c r="BH151" t="n">
         <v>1046.82474468344</v>
@@ -29028,13 +29028,13 @@
         <v>0.324984654635016</v>
       </c>
       <c r="BE152" t="n">
-        <v>2545.160555801388</v>
+        <v>2.545160555801389</v>
       </c>
       <c r="BF152" t="n">
-        <v>141426.1151832663</v>
+        <v>141.4261151832662</v>
       </c>
       <c r="BG152" t="n">
-        <v>94.21860149463978</v>
+        <v>0.09421860149463979</v>
       </c>
       <c r="BH152" t="n">
         <v>1501.04239438655</v>
@@ -29219,13 +29219,13 @@
         <v>0.4191162035677621</v>
       </c>
       <c r="BE153" t="n">
-        <v>2076.55949623921</v>
+        <v>2.07655949623921</v>
       </c>
       <c r="BF153" t="n">
-        <v>128140.3293853907</v>
+        <v>128.1403293853907</v>
       </c>
       <c r="BG153" t="n">
-        <v>114.6905287036673</v>
+        <v>0.1146905287036673</v>
       </c>
       <c r="BH153" t="n">
         <v>1117.270369521745</v>
@@ -29410,13 +29410,13 @@
         <v>0.4538509821073275</v>
       </c>
       <c r="BE154" t="n">
-        <v>2742.522983349366</v>
+        <v>2.742522983349367</v>
       </c>
       <c r="BF154" t="n">
-        <v>129647.9432373974</v>
+        <v>129.6479432373974</v>
       </c>
       <c r="BG154" t="n">
-        <v>123.1926864069352</v>
+        <v>0.1231926864069352</v>
       </c>
       <c r="BH154" t="n">
         <v>1052.399675814674</v>
@@ -29601,13 +29601,13 @@
         <v>0.7535500201908957</v>
       </c>
       <c r="BE155" t="n">
-        <v>2806.657621010977</v>
+        <v>2.806657621010977</v>
       </c>
       <c r="BF155" t="n">
-        <v>130790.8358063607</v>
+        <v>130.7908358063607</v>
       </c>
       <c r="BG155" t="n">
-        <v>207.4923530142719</v>
+        <v>0.2074923530142719</v>
       </c>
       <c r="BH155" t="n">
         <v>630.3405108975969</v>
@@ -29792,13 +29792,13 @@
         <v>1.172287562238779</v>
       </c>
       <c r="BE156" t="n">
-        <v>4003.25613157189</v>
+        <v>4.00325613157189</v>
       </c>
       <c r="BF156" t="n">
-        <v>145721.965743142</v>
+        <v>145.721965743142</v>
       </c>
       <c r="BG156" t="n">
-        <v>354.4257993513203</v>
+        <v>0.3544257993513203</v>
       </c>
       <c r="BH156" t="n">
         <v>411.1494310229285</v>
@@ -29983,13 +29983,13 @@
         <v>0.4231620695175342</v>
       </c>
       <c r="BE157" t="n">
-        <v>2615.744888154333</v>
+        <v>2.615744888154333</v>
       </c>
       <c r="BF157" t="n">
-        <v>145456.8526641889</v>
+        <v>145.4568526641889</v>
       </c>
       <c r="BG157" t="n">
-        <v>131.3219254796132</v>
+        <v>0.1313219254796132</v>
       </c>
       <c r="BH157" t="n">
         <v>1107.635698554923</v>
@@ -30174,13 +30174,13 @@
         <v>1.447062020901036</v>
       </c>
       <c r="BE158" t="n">
-        <v>3110.278188373693</v>
+        <v>3.110278188373694</v>
       </c>
       <c r="BF158" t="n">
-        <v>134120.3056081442</v>
+        <v>134.1203056081442</v>
       </c>
       <c r="BG158" t="n">
-        <v>392.9618776125638</v>
+        <v>0.3929618776125638</v>
       </c>
       <c r="BH158" t="n">
         <v>341.3061501614122</v>
@@ -30365,13 +30365,13 @@
         <v>1.447062020901036</v>
       </c>
       <c r="BE159" t="n">
-        <v>3110.278188373693</v>
+        <v>3.110278188373694</v>
       </c>
       <c r="BF159" t="n">
-        <v>134120.3056081442</v>
+        <v>134.1203056081442</v>
       </c>
       <c r="BG159" t="n">
-        <v>392.9618776125638</v>
+        <v>0.3929618776125638</v>
       </c>
       <c r="BH159" t="n">
         <v>341.3061501614122</v>
@@ -30556,13 +30556,13 @@
         <v>0.8361223093456559</v>
       </c>
       <c r="BE160" t="n">
-        <v>3178.492318378893</v>
+        <v>3.178492318378893</v>
       </c>
       <c r="BF160" t="n">
-        <v>129178.5542206582</v>
+        <v>129.1785542206582</v>
       </c>
       <c r="BG160" t="n">
-        <v>220.4215039302889</v>
+        <v>0.2204215039302889</v>
       </c>
       <c r="BH160" t="n">
         <v>586.052412842227</v>
@@ -30743,13 +30743,13 @@
         <v>0.8117757739071965</v>
       </c>
       <c r="BE161" t="n">
-        <v>3100.384113890322</v>
+        <v>3.100384113890322</v>
       </c>
       <c r="BF161" t="n">
-        <v>123593.3624024007</v>
+        <v>123.5933624024007</v>
       </c>
       <c r="BG161" t="n">
-        <v>203.8814339992062</v>
+        <v>0.2038814339992062</v>
       </c>
       <c r="BH161" t="n">
         <v>606.2021439523618</v>
@@ -30930,13 +30930,13 @@
         <v>0.5765357094251896</v>
       </c>
       <c r="BE162" t="n">
-        <v>2368.124449995078</v>
+        <v>2.368124449995078</v>
       </c>
       <c r="BF162" t="n">
-        <v>119565.5202168899</v>
+        <v>119.5655202168899</v>
       </c>
       <c r="BG162" t="n">
-        <v>147.8461330180165</v>
+        <v>0.1478461330180165</v>
       </c>
       <c r="BH162" t="n">
         <v>808.7159114423353</v>
@@ -31121,13 +31121,13 @@
         <v>1.046102945540786</v>
       </c>
       <c r="BE163" t="n">
-        <v>2494.800680792413</v>
+        <v>2.494800680792413</v>
       </c>
       <c r="BF163" t="n">
-        <v>132442.1082301923</v>
+        <v>132.4421082301923</v>
       </c>
       <c r="BG163" t="n">
-        <v>298.7919429514647</v>
+        <v>0.2987919429514647</v>
       </c>
       <c r="BH163" t="n">
         <v>443.2586331543284</v>
@@ -31312,13 +31312,13 @@
         <v>0.4695082726749009</v>
       </c>
       <c r="BE164" t="n">
-        <v>2936.607957022901</v>
+        <v>2.936607957022901</v>
       </c>
       <c r="BF164" t="n">
-        <v>132735.0949602475</v>
+        <v>132.7350949602475</v>
       </c>
       <c r="BG164" t="n">
-        <v>131.2849522275966</v>
+        <v>0.1312849522275966</v>
       </c>
       <c r="BH164" t="n">
         <v>1011.045765017585</v>
@@ -31503,13 +31503,13 @@
         <v>1.240984290338432</v>
       </c>
       <c r="BE165" t="n">
-        <v>2706.029629235518</v>
+        <v>2.706029629235518</v>
       </c>
       <c r="BF165" t="n">
-        <v>130340.932329563</v>
+        <v>130.340932329563</v>
       </c>
       <c r="BG165" t="n">
-        <v>344.2185085599922</v>
+        <v>0.3442185085599922</v>
       </c>
       <c r="BH165" t="n">
         <v>378.6575360948277</v>
@@ -31694,13 +31694,13 @@
         <v>1.507902613849702</v>
       </c>
       <c r="BE166" t="n">
-        <v>4035.463229976435</v>
+        <v>4.035463229976434</v>
       </c>
       <c r="BF166" t="n">
-        <v>171968.2607603812</v>
+        <v>171.9682607603812</v>
       </c>
       <c r="BG166" t="n">
-        <v>515.1927582473124</v>
+        <v>0.5151927582473125</v>
       </c>
       <c r="BH166" t="n">
         <v>333.794017884525</v>
@@ -31885,13 +31885,13 @@
         <v>1.110726579043297</v>
       </c>
       <c r="BE167" t="n">
-        <v>2808.389842928612</v>
+        <v>2.808389842928612</v>
       </c>
       <c r="BF167" t="n">
-        <v>119272.127037589</v>
+        <v>119.272127037589</v>
       </c>
       <c r="BG167" t="n">
-        <v>275.5068721173976</v>
+        <v>0.2755068721173976</v>
       </c>
       <c r="BH167" t="n">
         <v>432.9188819172734</v>
@@ -32076,13 +32076,13 @@
         <v>0.7129588548014306</v>
       </c>
       <c r="BE168" t="n">
-        <v>3925.394607703596</v>
+        <v>3.925394607703596</v>
       </c>
       <c r="BF168" t="n">
-        <v>150762.6863250885</v>
+        <v>150.7626863250885</v>
       </c>
       <c r="BG168" t="n">
-        <v>216.3390994957416</v>
+        <v>0.2163390994957415</v>
       </c>
       <c r="BH168" t="n">
         <v>696.8813620676838</v>
@@ -32267,13 +32267,13 @@
         <v>0.7458032085161251</v>
       </c>
       <c r="BE169" t="n">
-        <v>3010.46998120762</v>
+        <v>3.01046998120762</v>
       </c>
       <c r="BF169" t="n">
-        <v>124271.211508699</v>
+        <v>124.271211508699</v>
       </c>
       <c r="BG169" t="n">
-        <v>197.3079548330844</v>
+        <v>0.1973079548330844</v>
       </c>
       <c r="BH169" t="n">
         <v>629.8337622212349</v>
@@ -32458,13 +32458,13 @@
         <v>1.060681081061475</v>
       </c>
       <c r="BE170" t="n">
-        <v>3857.753490063654</v>
+        <v>3.857753490063654</v>
       </c>
       <c r="BF170" t="n">
-        <v>156769.4106261306</v>
+        <v>156.7694106261306</v>
       </c>
       <c r="BG170" t="n">
-        <v>333.7167716726452</v>
+        <v>0.3337167716726452</v>
       </c>
       <c r="BH170" t="n">
         <v>469.7678508645989</v>
@@ -32649,13 +32649,13 @@
         <v>0.876007634737751</v>
       </c>
       <c r="BE171" t="n">
-        <v>3060.13376015371</v>
+        <v>3.06013376015371</v>
       </c>
       <c r="BF171" t="n">
-        <v>116550.839363781</v>
+        <v>116.550839363781</v>
       </c>
       <c r="BG171" t="n">
-        <v>210.4132050197028</v>
+        <v>0.2104132050197028</v>
       </c>
       <c r="BH171" t="n">
         <v>553.914091812191</v>
@@ -32840,13 +32840,13 @@
         <v>0.7321314863248521</v>
       </c>
       <c r="BE172" t="n">
-        <v>3580.328574778584</v>
+        <v>3.580328574778584</v>
       </c>
       <c r="BF172" t="n">
-        <v>155139.5166682314</v>
+        <v>155.1395166682314</v>
       </c>
       <c r="BG172" t="n">
-        <v>227.9105775244651</v>
+        <v>0.2279105775244651</v>
       </c>
       <c r="BH172" t="n">
         <v>680.7034511225257</v>
@@ -33031,13 +33031,13 @@
         <v>0.7135182431806696</v>
       </c>
       <c r="BE173" t="n">
-        <v>2714.433523098972</v>
+        <v>2.714433523098972</v>
       </c>
       <c r="BF173" t="n">
-        <v>123772.2705281614</v>
+        <v>123.7722705281614</v>
       </c>
       <c r="BG173" t="n">
-        <v>182.5892575668475</v>
+        <v>0.1825892575668475</v>
       </c>
       <c r="BH173" t="n">
         <v>677.8726863646251</v>
@@ -33222,13 +33222,13 @@
         <v>0.4657407982928221</v>
       </c>
       <c r="BE174" t="n">
-        <v>2969.412381357694</v>
+        <v>2.969412381357694</v>
       </c>
       <c r="BF174" t="n">
-        <v>136856.1441562886</v>
+        <v>136.8561441562886</v>
       </c>
       <c r="BG174" t="n">
-        <v>135.0134270421117</v>
+        <v>0.1350134270421117</v>
       </c>
       <c r="BH174" t="n">
         <v>1013.648398937405</v>
@@ -33413,13 +33413,13 @@
         <v>1.076097980645826</v>
       </c>
       <c r="BE175" t="n">
-        <v>3590.220428377389</v>
+        <v>3.590220428377389</v>
       </c>
       <c r="BF175" t="n">
-        <v>112022.7161869101</v>
+        <v>112.0227161869101</v>
       </c>
       <c r="BG175" t="n">
-        <v>247.3438134994981</v>
+        <v>0.2473438134994981</v>
       </c>
       <c r="BH175" t="n">
         <v>452.9028424118535</v>
@@ -33604,13 +33604,13 @@
         <v>0.7889988860287893</v>
       </c>
       <c r="BE176" t="n">
-        <v>3145.971770441211</v>
+        <v>3.145971770441211</v>
       </c>
       <c r="BF176" t="n">
-        <v>117900.075239499</v>
+        <v>117.900075239499</v>
       </c>
       <c r="BG176" t="n">
-        <v>189.2709314371093</v>
+        <v>0.1892709314371092</v>
       </c>
       <c r="BH176" t="n">
         <v>622.9169706319891</v>
@@ -33795,13 +33795,13 @@
         <v>0.8998972351497689</v>
       </c>
       <c r="BE177" t="n">
-        <v>2988.045897731698</v>
+        <v>2.988045897731697</v>
       </c>
       <c r="BF177" t="n">
-        <v>137153.0243619897</v>
+        <v>137.1530243619897</v>
       </c>
       <c r="BG177" t="n">
-        <v>250.1943599445277</v>
+        <v>0.2501943599445277</v>
       </c>
       <c r="BH177" t="n">
         <v>548.1859159111293</v>
@@ -33986,13 +33986,13 @@
         <v>0.760049464742248</v>
       </c>
       <c r="BE178" t="n">
-        <v>2795.080671498331</v>
+        <v>2.795080671498331</v>
       </c>
       <c r="BF178" t="n">
-        <v>132491.1744332169</v>
+        <v>132.4911744332169</v>
       </c>
       <c r="BG178" t="n">
-        <v>221.1978616315913</v>
+        <v>0.2211978616315912</v>
       </c>
       <c r="BH178" t="n">
         <v>598.971316702343</v>
@@ -34177,13 +34177,13 @@
         <v>0.8704905427894011</v>
       </c>
       <c r="BE179" t="n">
-        <v>2991.504895299842</v>
+        <v>2.991504895299842</v>
       </c>
       <c r="BF179" t="n">
-        <v>133846.1268133776</v>
+        <v>133.8461268133776</v>
       </c>
       <c r="BG179" t="n">
-        <v>246.3050873924967</v>
+        <v>0.2463050873924967</v>
       </c>
       <c r="BH179" t="n">
         <v>543.4160058581681</v>
@@ -34368,13 +34368,13 @@
         <v>0.7904204876191047</v>
       </c>
       <c r="BE180" t="n">
-        <v>2715.490388769533</v>
+        <v>2.715490388769533</v>
       </c>
       <c r="BF180" t="n">
-        <v>119574.7805559971</v>
+        <v>119.5747805559971</v>
       </c>
       <c r="BG180" t="n">
-        <v>204.5078913327457</v>
+        <v>0.2045078913327457</v>
       </c>
       <c r="BH180" t="n">
         <v>584.6951908640156</v>
@@ -34559,13 +34559,13 @@
         <v>0.4290615053355752</v>
       </c>
       <c r="BE181" t="n">
-        <v>2886.034344314457</v>
+        <v>2.886034344314457</v>
       </c>
       <c r="BF181" t="n">
-        <v>156425.1632215068</v>
+        <v>156.4251632215068</v>
       </c>
       <c r="BG181" t="n">
-        <v>142.1757845401308</v>
+        <v>0.1421757845401308</v>
       </c>
       <c r="BH181" t="n">
         <v>1100.223668379716</v>
@@ -34750,13 +34750,13 @@
         <v>0.8868190945788528</v>
       </c>
       <c r="BE182" t="n">
-        <v>3227.764288178313</v>
+        <v>3.227764288178313</v>
       </c>
       <c r="BF182" t="n">
-        <v>127135.1919261465</v>
+        <v>127.1351919261465</v>
       </c>
       <c r="BG182" t="n">
-        <v>225.7504469348979</v>
+        <v>0.2257504469348978</v>
       </c>
       <c r="BH182" t="n">
         <v>563.1669556021295</v>
@@ -34941,13 +34941,13 @@
         <v>0.579333851742069</v>
       </c>
       <c r="BE183" t="n">
-        <v>2924.394554936031</v>
+        <v>2.924394554936031</v>
       </c>
       <c r="BF183" t="n">
-        <v>125114.0993119449</v>
+        <v>125.1140993119449</v>
       </c>
       <c r="BG183" t="n">
-        <v>157.6035535331282</v>
+        <v>0.1576035535331282</v>
       </c>
       <c r="BH183" t="n">
         <v>793.8532888831468</v>

</xml_diff>